<commit_message>
fix(excel): Antes de este commit funcionaba indivudal y consolidado con pequeños errores al compilar el xml
</commit_message>
<xml_diff>
--- a/scripts/.tmp/audit-cons.xlsx
+++ b/scripts/.tmp/audit-cons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Documents\proyecto_cursor\proyectoisaqwenvisor\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49775DE-810D-4758-A059-F713516FBF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD33005-EBB4-4B92-8E86-6A1E6A6B1D7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -1021,7 +1021,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="220">
+  <cellXfs count="219">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1109,9 +1109,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="42" fontId="6" fillId="0" borderId="25" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1450,164 +1447,164 @@
     <xf numFmtId="42" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="42" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="18" fillId="4" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1949,6 +1946,3021 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac xr xr2 xr3" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{00000000-0001-0000-0000-000000000000}"><dimension ref="A1:W145"/><sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/><cols><col min="1" max="1" width="17.33203125" customWidth="1"/><col min="2" max="2" width="13.88671875" style="1" bestFit="1" customWidth="1"/><col min="3" max="3" width="12.6640625" customWidth="1"/><col min="4" max="4" width="12.6640625" style="3" customWidth="1"/><col min="5" max="5" width="12.6640625" customWidth="1"/><col min="6" max="6" width="12.6640625" style="3" customWidth="1"/><col min="7" max="9" width="12.6640625" customWidth="1"/><col min="10" max="10" width="12.6640625" style="3" customWidth="1"/><col min="11" max="11" width="12.6640625" customWidth="1"/><col min="12" max="12" width="12.6640625" style="3" customWidth="1"/><col min="13" max="13" width="11.5546875" style="3" customWidth="1"/><col min="14" max="14" width="11" bestFit="1" customWidth="1"/><col min="15" max="15" width="11.6640625" style="4" customWidth="1"/><col min="16" max="19" width="11.6640625" style="3" customWidth="1"/><col min="20" max="20" width="13.88671875" customWidth="1"/><col min="21" max="21" width="14" customWidth="1"/><col min="22" max="22" width="19.33203125" bestFit="1" customWidth="1"/><col min="23" max="23" width="16" customWidth="1"/></cols><sheetData><row r="1" spans="1:23" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"><c r="A1" s="7" t="s"><v>50</v></c><c r="B1" s="112" t="inlineStr"><is><t xml:space="preserve">CRISTIAN</t></is></c><c r="C1" s="120" t="inlineStr"><is><t xml:space="preserve">CRISTIAN</t></is></c><c r="D1" s="120" t="inlineStr"><is><t xml:space="preserve">PEDRO</t></is></c><c r="E1" s="112"/><c r="F1" s="120"/><c r="G1" s="120"/><c r="H1" s="112"/><c r="I1" s="112"/><c r="J1" s="120"/><c r="K1" s="120"/><c r="L1" s="112"/><c r="M1" s="112"/><c r="N1" s="112"/><c r="O1" s="112"/><c r="P1" s="112"/><c r="Q1" s="112"/><c r="R1" s="121"/><c r="S1" s="120"/><c r="T1" s="120"/><c r="U1" s="7"/><c r="V1" s="7"/><c r="W1" s="114"/></row><row r="2" spans="1:23" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"><c r="A2" s="7" t="s"><v>51</v></c><c r="B2" s="112"/><c r="C2" s="120"/><c r="D2" s="120"/><c r="E2" s="112"/><c r="F2" s="120"/><c r="G2" s="128"/><c r="H2" s="112"/><c r="I2" s="112"/><c r="J2" s="120"/><c r="K2" s="120"/><c r="L2" s="112"/><c r="M2" s="112"/><c r="N2" s="112"/><c r="O2" s="112"/><c r="P2" s="112"/><c r="Q2" s="112"/><c r="R2" s="121"/><c r="S2" s="120"/><c r="T2" s="120"/><c r="U2" s="7"/><c r="V2" s="7"/><c r="W2" s="114"/></row><row r="3" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A3" s="122" t="s"><v>35</v></c><c r="B3" s="120"/><c r="C3" s="120"/><c r="D3" s="120"/><c r="E3" s="120"/><c r="F3" s="120"/><c r="G3" s="120"/><c r="H3" s="120"/><c r="I3" s="120"/><c r="J3" s="120"/><c r="K3" s="120"/><c r="L3" s="120"/><c r="M3" s="120"/><c r="N3" s="120"/><c r="O3" s="120"/><c r="P3" s="120"/><c r="Q3" s="120"/><c r="R3" s="120"/><c r="S3" s="120"/><c r="T3" s="120"/><c r="U3" s="110"/><c r="V3" s="163"/><c r="W3" s="116"/></row><row r="4" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A4" s="122" t="s"><v>52</v></c><c r="B4" s="120"/><c r="C4" s="120"/><c r="D4" s="120"/><c r="E4" s="120"/><c r="F4" s="120"/><c r="G4" s="120"/><c r="H4" s="120"/><c r="I4" s="120"/><c r="J4" s="120"/><c r="K4" s="120"/><c r="L4" s="120"/><c r="M4" s="120"/><c r="N4" s="120"/><c r="O4" s="120"/><c r="P4" s="120"/><c r="Q4" s="120"/><c r="R4" s="120"/><c r="S4" s="120"/><c r="T4" s="120"/><c r="U4" s="110"/><c r="V4" s="163"/><c r="W4" s="116"/></row><row r="5" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A5" s="122" t="s"><v>0</v></c><c r="B5" s="129" t="inlineStr"><is><t xml:space="preserve">260006341</t></is></c><c r="C5" s="129" t="inlineStr"><is><t xml:space="preserve">260006342</t></is></c><c r="D5" s="129" t="inlineStr"><is><t xml:space="preserve">260006320</t></is></c><c r="E5" s="129"/><c r="F5" s="129"/><c r="G5" s="129"/><c r="H5" s="129"/><c r="I5" s="129"/><c r="J5" s="129"/><c r="K5" s="129"/><c r="L5" s="129"/><c r="M5" s="129"/><c r="N5" s="129"/><c r="O5" s="129"/><c r="P5" s="129"/><c r="Q5" s="129"/><c r="R5" s="120"/><c r="S5" s="120"/><c r="T5" s="120"/><c r="U5" s="111"/><c r="V5" s="111"/><c r="W5" s="111"/></row><row r="6" spans="1:23" s="45" customFormat="1" x14ac:dyDescent="0.3"><c r="A6" s="122" t="s"><v>1</v></c><c r="B6" s="120"><v>5</v></c><c r="C6" s="120"><v>5</v></c><c r="D6" s="120"><v>5</v></c><c r="E6" s="120"/><c r="F6" s="120"/><c r="G6" s="120"/><c r="H6" s="120"/><c r="I6" s="120"/><c r="J6" s="120"/><c r="K6" s="120"/><c r="L6" s="120"/><c r="M6" s="111"/><c r="N6" s="111"/><c r="O6" s="111"/><c r="P6" s="111"/><c r="Q6" s="111"/><c r="R6" s="120"/><c r="S6" s="120"/><c r="T6" s="120"/><c r="U6" s="111"/><c r="V6" s="111"/><c r="W6" s="111"/></row><row r="7" spans="1:23" s="45" customFormat="1" ht="72" x14ac:dyDescent="0.3"><c r="A7" s="122" t="s"><v>2</v></c><c r="B7" s="164"><v>1000000</v></c><c r="C7" s="164"><v>1000000</v></c><c r="D7" s="164"><v>1054260</v></c><c r="E7" s="164"/><c r="F7" s="164"/><c r="G7" s="164"/><c r="H7" s="164"/><c r="I7" s="164"/><c r="J7" s="164"/><c r="K7" s="164"/><c r="L7" s="164"/><c r="M7" s="164"/><c r="N7" s="164"/><c r="O7" s="164"/><c r="P7" s="164"/><c r="Q7" s="164"/><c r="R7" s="156"/><c r="S7" s="156"/><c r="T7" s="156"/><c r="U7" s="157"/><c r="V7" s="157"/><c r="W7" s="157"/></row><row r="8" spans="1:23" s="45" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A8" s="112"/><c r="B8" s="157"/><c r="C8" s="111"/><c r="D8" s="157"/><c r="E8" s="111"/><c r="F8" s="110"/><c r="G8" s="111"/><c r="H8" s="157"/><c r="I8" s="111"/><c r="J8" s="157"/><c r="K8" s="111"/><c r="L8" s="110"/><c r="M8" s="111"/><c r="N8" s="110"/><c r="O8" s="111"/><c r="P8" s="158"/><c r="Q8" s="111"/><c r="R8" s="158"/><c r="S8" s="111"/><c r="T8" s="158"/><c r="U8" s="111"/><c r="V8" s="110"/><c r="W8" s="111"/></row><row r="9" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A9" s="113" t="s"><v>3</v></c><c r="B9" s="165"/><c r="C9" s="165"/><c r="D9" s="165"/><c r="E9" s="157"/><c r="F9" s="110"/><c r="G9" s="157"/><c r="H9" s="110"/><c r="I9" s="157"/><c r="J9" s="110"/><c r="K9" s="157"/><c r="L9" s="110"/><c r="M9" s="157"/><c r="N9" s="110"/><c r="O9" s="157"/><c r="P9" s="158"/><c r="Q9" s="157"/><c r="R9" s="158"/><c r="S9" s="159"/><c r="T9" s="159"/><c r="U9" s="157"/><c r="V9" s="110"/><c r="W9" s="157"/></row><row r="10" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A10" s="113" t="s"><v>54</v></c><c r="B10" s="165"/><c r="C10" s="165"/><c r="D10" s="165"/><c r="E10" s="157"/><c r="F10" s="110"/><c r="G10" s="157"/><c r="H10" s="110"/><c r="I10" s="157"/><c r="J10" s="110"/><c r="K10" s="157"/><c r="L10" s="110"/><c r="M10" s="157"/><c r="N10" s="110"/><c r="O10" s="157"/><c r="P10" s="158"/><c r="Q10" s="157"/><c r="R10" s="158"/><c r="S10" s="159"/><c r="T10" s="159"/><c r="U10" s="157"/><c r="V10" s="110"/><c r="W10" s="157"/></row><row r="11" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A11" s="113" t="s"><v>4</v></c><c r="B11" s="165"/><c r="C11" s="165"/><c r="D11" s="165"/><c r="E11" s="157"/><c r="F11" s="110"/><c r="G11" s="157"/><c r="H11" s="110"/><c r="I11" s="157"/><c r="J11" s="110"/><c r="K11" s="157"/><c r="L11" s="110"/><c r="M11" s="157"/><c r="N11" s="110"/><c r="O11" s="157"/><c r="P11" s="158"/><c r="Q11" s="157"/><c r="R11" s="158"/><c r="S11" s="159"/><c r="T11" s="159"/><c r="U11" s="157"/><c r="V11" s="110"/><c r="W11" s="157"/></row><row r="12" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A12" s="113" t="s"><v>5</v></c><c r="B12" s="165"><v>127092</v></c><c r="C12" s="165"><v>972618</v></c><c r="D12" s="165"><v>461001</v></c><c r="E12" s="157"/><c r="F12" s="110"/><c r="G12" s="157"/><c r="H12" s="110"/><c r="I12" s="157"/><c r="J12" s="110"/><c r="K12" s="157"/><c r="L12" s="110"/><c r="M12" s="157"/><c r="N12" s="110"/><c r="O12" s="157"/><c r="P12" s="158"/><c r="Q12" s="157"/><c r="R12" s="158"/><c r="S12" s="159"/><c r="T12" s="159"/><c r="U12" s="157"/><c r="V12" s="110"/><c r="W12" s="157"/></row><row r="13" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A13" s="113" t="s"><v>6</v></c><c r="B13" s="165"/><c r="C13" s="165"/><c r="D13" s="165"/><c r="E13" s="157"/><c r="F13" s="110"/><c r="G13" s="157"/><c r="H13" s="110"/><c r="I13" s="157"/><c r="J13" s="110"/><c r="K13" s="157"/><c r="L13" s="110"/><c r="M13" s="157"/><c r="N13" s="110"/><c r="O13" s="157"/><c r="P13" s="158"/><c r="Q13" s="157"/><c r="R13" s="158"/><c r="S13" s="159"/><c r="T13" s="159"/><c r="U13" s="157"/><c r="V13" s="110"/><c r="W13" s="157"/></row><row r="14" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A14" s="113" t="s"><v>7</v></c><c r="B14" s="165"/><c r="C14" s="165"/><c r="D14" s="165"/><c r="E14" s="157"/><c r="F14" s="110"/><c r="G14" s="157"/><c r="H14" s="110"/><c r="I14" s="157"/><c r="J14" s="110"/><c r="K14" s="157"/><c r="L14" s="110"/><c r="M14" s="157"/><c r="N14" s="110"/><c r="O14" s="157"/><c r="P14" s="158"/><c r="Q14" s="157"/><c r="R14" s="158"/><c r="S14" s="159"/><c r="T14" s="159"/><c r="U14" s="157"/><c r="V14" s="110"/><c r="W14" s="157"/></row><row r="15" spans="1:23" s="161" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"><c r="A15" s="113" t="s"><v>8</v></c><c r="B15" s="165"/><c r="C15" s="165"/><c r="D15" s="165"/><c r="E15" s="157"/><c r="F15" s="110"/><c r="G15" s="157"/><c r="H15" s="110"/><c r="I15" s="157"/><c r="J15" s="110"/><c r="K15" s="157"/><c r="L15" s="110"/><c r="M15" s="157"/><c r="N15" s="110"/><c r="O15" s="157"/><c r="P15" s="158"/><c r="Q15" s="157"/><c r="R15" s="158"/><c r="S15" s="159"/><c r="T15" s="159"/><c r="U15" s="157"/><c r="V15" s="110"/><c r="W15" s="157"/></row><row r="16" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3"><c r="A16" s="113" t="s"><v>9</v></c><c r="B16" s="165"/><c r="C16" s="165"/><c r="D16" s="165"/><c r="E16" s="157"/><c r="F16" s="110"/><c r="G16" s="157"/><c r="H16" s="110"/><c r="I16" s="160"/><c r="J16" s="110"/><c r="K16" s="160"/><c r="L16" s="110"/><c r="M16" s="157"/><c r="N16" s="110"/><c r="O16" s="157"/><c r="P16" s="158"/><c r="Q16" s="157"/><c r="R16" s="158"/><c r="S16" s="159"/><c r="T16" s="159"/><c r="U16" s="157"/><c r="V16" s="110"/><c r="W16" s="157"/></row><row r="17" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3"><c r="A17" s="113" t="s"><v>10</v></c><c r="B17" s="165"/><c r="C17" s="165"/><c r="D17" s="165"/><c r="E17" s="157"/><c r="F17" s="110"/><c r="G17" s="157"/><c r="H17" s="110"/><c r="I17" s="160"/><c r="J17" s="110"/><c r="K17" s="157"/><c r="L17" s="110"/><c r="M17" s="157"/><c r="N17" s="110"/><c r="O17" s="157"/><c r="P17" s="158"/><c r="Q17" s="157"/><c r="R17" s="158"/><c r="S17" s="159"/><c r="T17" s="159"/><c r="U17" s="157"/><c r="V17" s="110"/><c r="W17" s="157"/></row><row r="18" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3"><c r="A18" s="113" t="s"><v>11</v></c><c r="B18" s="110"><f>SUM(B9:B17)</f><v>0</v></c><c r="C18" s="110"><f t="shared" ref="C18:O18" si="0">SUM(C9:C17)</f><v>0</v></c><c r="D18" s="110"><f t="shared" si="0"/><c r="E18" s="110"><f t="shared" si="0"/><c r="F18" s="110"><f t="shared" si="0"/><c r="G18" s="110"><f t="shared" si="0"/><c r="H18" s="110"><f t="shared" si="0"/><c r="I18" s="110"><f t="shared" si="0"/><c r="J18" s="110"><f t="shared" si="0"/><c r="K18" s="110"><f t="shared" si="0"/><c r="L18" s="110"><f t="shared" si="0"/><c r="M18" s="110"><f t="shared" si="0"/><c r="N18" s="110"><f t="shared" si="0"/><c r="O18" s="110"><f t="shared" si="0"/><c r="P18" s="110"><f t="shared" ref="P18" si="1">SUM(P9:P17)</f><v>0</v></c><c r="Q18" s="110"><f>SUM(Q9:Q17)</f><v>0</v></c><c r="R18" s="110"><f>SUM(R9:R17)</f><v>0</v></c><c r="S18" s="116"><f>SUM(S9:S17)</f><v>0</v></c><c r="T18" s="116"><f>SUM(T9:T17)</f><v>0</v></c><c r="U18" s="110"><f t="shared" ref="U18:W18" si="2">SUM(U9:U17)</f><v>0</v></c><c r="V18" s="110"><f t="shared" si="2"/><c r="W18" s="110"><f t="shared" si="2"/></row><row r="19" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3"><c r="A19" s="113"/><c r="B19" s="110"/><c r="C19" s="110"/><c r="D19" s="110"/><c r="E19" s="110"/><c r="F19" s="157"/><c r="G19" s="110"/><c r="H19" s="110"/><c r="I19" s="110"/><c r="J19" s="110"/><c r="K19" s="110"/><c r="L19" s="110"/><c r="M19" s="110"/><c r="N19" s="110"/><c r="O19" s="110"/><c r="P19" s="110"/><c r="Q19" s="110"/><c r="R19" s="110"/><c r="S19" s="116"/><c r="T19" s="116"/><c r="U19" s="110"/><c r="V19" s="110"/><c r="W19" s="110"/></row><row r="20" spans="1:23" s="162" customFormat="1" x14ac:dyDescent="0.3"><c r="A20" s="113" t="s"><v>12</v></c><c r="B20" s="110" t="e"><f t="shared" ref="B20:O20" si="3">B18-B7</f><v>#VALUE!</v></c><c r="C20" s="110"><f t="shared" si="3"/><c r="D20" s="110"><f t="shared" si="3"/><c r="E20" s="110"><f t="shared" si="3"/><c r="F20" s="110"><f t="shared" si="3"/><c r="G20" s="110"><f t="shared" si="3"/><c r="H20" s="110"><f t="shared" si="3"/><c r="I20" s="110"><f t="shared" si="3"/><c r="J20" s="110"><f t="shared" si="3"/><c r="K20" s="110"><f t="shared" si="3"/><c r="L20" s="110"><f t="shared" si="3"/><c r="M20" s="110"><f t="shared" si="3"/><c r="N20" s="110"><f t="shared" si="3"/><c r="O20" s="110"><f t="shared" si="3"/><c r="P20" s="110"><f t="shared" ref="P20" si="4">P18-P7</f><v>0</v></c><c r="Q20" s="110"><f>Q18-Q7</f><v>0</v></c><c r="R20" s="110"><f>R18-R7</f><v>0</v></c><c r="S20" s="110"><f>S18-S7</f><v>0</v></c><c r="T20" s="110"><f>T18-T7</f><v>0</v></c><c r="U20" s="110"><f t="shared" ref="U20:W20" si="5">U18-U7</f><v>0</v></c><c r="V20" s="110"><f t="shared" si="5"/><c r="W20" s="110"><f t="shared" si="5"/></row><row r="21" spans="1:23" x14ac:dyDescent="0.3"><c r="A21" s="1"/><c r="B21" s="9"/><c r="C21" s="10"/><c r="D21" s="9"/><c r="E21" s="10"/><c r="F21" s="11"/><c r="G21" s="10"/><c r="H21" s="11"/><c r="I21" s="9"/><c r="J21" s="9"/><c r="K21" s="10"/><c r="L21" s="12"/><c r="M21" s="12"/><c r="N21" s="10"/><c r="O21" s="9"/><c r="P21" s="9"/><c r="Q21" s="10"/><c r="R21" s="12"/><c r="S21" s="12"/><c r="T21" s="9"/><c r="U21" s="9"/><c r="V21" s="9"/><c r="W21" s="9"/></row><row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35"><c r="D22" s="2"/><c r="M22" s="198" t="s"><v>48</v></c><c r="N22" s="198"/><c r="O22" s="198"/><c r="P22" s="198"/><c r="Q22" s="198"/><c r="R22" s="198"/><c r="S22" s="198"/><c r="T22" s="198"/><c r="U22" s="198"/></row><row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"><c r="D23" s="6"/><c r="J23"/><c r="L23"/><c r="M23" s="14" t="s"><v>13</v></c><c r="N23" s="207" t="inlineStr"><is><t xml:space="preserve">30-06-2026</t></is></c><c r="O23" s="208"/><c r="P23" s="208"/><c r="Q23" s="208"/><c r="R23" s="208"/><c r="S23" s="209"/><c r="T23" s="119" t="s"><v>38</v></c><c r="U23" s="106"><v>15</v></c><c r="W23" s="91" t="s"><v>44</v></c></row><row r="24" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"><c r="B24" s="2"/><c r="C24" s="18"/><c r="J24"/><c r="K24" s="15"/><c r="L24"/><c r="M24" s="16"/><c r="N24" s="210" t="s"><v>49</v></c><c r="O24" s="211"/><c r="P24" s="211"/><c r="Q24" s="211"/><c r="R24" s="211"/><c r="S24" s="212"/><c r="T24" s="108" t="s"><v>11</v></c><c r="U24" s="107"><v>3054260</v></c><c r="W24" s="118"><v>15</v></c></row><row r="25" spans="1:23" x14ac:dyDescent="0.3"><c r="B25" s="2"/><c r="C25" s="103"/><c r="D25" s="3" t="s"><v>15</v></c><c r="E25" s="4"/><c r="J25"/><c r="L25"/><c r="M25" s="215" t="s"><v>16</v></c><c r="N25" s="216"/><c r="O25" s="148"/><c r="P25" s="149"/><c r="Q25" s="145"/><c r="R25" s="146"/><c r="S25" s="147"/><c r="T25" s="213" t="s"><v>17</v></c><c r="U25" s="214"/><c r="V25" s="13"/><c r="W25" s="82" t="s"><v>45</v></c></row><row r="26" spans="1:23" x14ac:dyDescent="0.3"><c r="E26" s="4"/><c r="J26"/><c r="L26"/><c r="M26" s="79" t="s"><v>53</v></c><c r="N26" s="80"/><c r="O26" s="126"/><c r="P26" s="127"/><c r="Q26" s="188"/><c r="R26" s="189"/><c r="S26" s="190"/><c r="T26" s="124"/><c r="U26" s="125"/><c r="V26" s="13"/><c r="W26" s="82"/></row><row r="27" spans="1:23" x14ac:dyDescent="0.3"><c r="I27" s="109" t="str"><f>B1</f></c><c r="J27" s="136" t="str"><f>B9</f></c><c r="L27"/><c r="M27" s="79" t="s"><v>18</v></c><c r="N27" s="80"/><c r="O27" s="186"/><c r="P27" s="187"/><c r="Q27" s="188"/><c r="R27" s="189"/><c r="S27" s="190"/><c r="T27" s="205" t="s"><v>19</v></c><c r="U27" s="206"/><c r="V27" s="19"/><c r="W27" s="92"><v>3054260</v></c></row><row r="28" spans="1:23" x14ac:dyDescent="0.3"><c r="I28" s="109"><f>C1</f><v>0</v></c><c r="J28" s="136"><f>C9</f><v>0</v></c><c r="L28"/><c r="M28" s="203" t="s"><v>20</v></c><c r="N28" s="204"/><c r="O28" s="186"/><c r="P28" s="187"/><c r="Q28" s="188"><v>1560711</v></c><c r="R28" s="189"/><c r="S28" s="190"/><c r="T28" s="201" t="s"><v>39</v></c><c r="U28" s="202"/><c r="V28" s="21"/><c r="W28" s="13"/></row><row r="29" spans="1:23" x14ac:dyDescent="0.3"><c r="I29" s="109"><f>D1</f><v>0</v></c><c r="J29" s="136"><f>D9</f><v>0</v></c><c r="K29" s="24"/><c r="L29"/><c r="M29" s="203" t="s"><v>21</v></c><c r="N29" s="204"/><c r="O29" s="186"/><c r="P29" s="187"/><c r="Q29" s="188"/><c r="R29" s="189"/><c r="S29" s="190"/><c r="T29" s="199" t="s"><v>40</v></c><c r="U29" s="200"/><c r="W29" s="93" t="str"><f>U23</f></c></row><row r="30" spans="1:23" x14ac:dyDescent="0.3"><c r="A30" s="1"/><c r="I30" s="109"><f>E1</f><v>0</v></c><c r="J30" s="136"><f>E9</f><v>0</v></c><c r="L30"/><c r="M30" s="203" t="s"><v>22</v></c><c r="N30" s="204"/><c r="O30" s="186"/><c r="P30" s="217"/><c r="Q30" s="188"/><c r="R30" s="189"/><c r="S30" s="190"/><c r="T30" s="218" t="s"><v>41</v></c><c r="U30" s="219"/><c r="V30" s="24"/><c r="W30" s="21" t="str"><f>Q34</f></c></row><row r="31" spans="1:23" x14ac:dyDescent="0.3"><c r="A31" s="1"/><c r="I31" s="109"><f>F1</f><v>0</v></c><c r="J31" s="136"><f>F9</f><v>0</v></c><c r="L31"/><c r="M31" s="203" t="s"><v>23</v></c><c r="N31" s="204"/><c r="O31" s="186"/><c r="P31" s="187"/><c r="Q31" s="188"/><c r="R31" s="189"/><c r="S31" s="190"/><c r="T31" s="28"/><c r="U31" s="26"/></row><row r="32" spans="1:23" x14ac:dyDescent="0.3"><c r="A32" s="1"/><c r="I32" s="109"><f>G1</f><v>0</v></c><c r="J32" s="136"><f>G9</f><v>0</v></c><c r="L32"/><c r="M32" s="203" t="s"><v>24</v></c><c r="N32" s="204"/><c r="O32" s="186"/><c r="P32" s="187"/><c r="Q32" s="188"/><c r="R32" s="189"/><c r="S32" s="190"/><c r="T32" s="28"/><c r="U32" s="26"/><c r="W32" s="82" t="s"><v>46</v></c></row><row r="33" spans="1:23" x14ac:dyDescent="0.3"><c r="A33" s="1"/><c r="I33" s="109"><f>H1</f><v>0</v></c><c r="J33" s="136"><f>H9</f><v>0</v></c><c r="L33"/><c r="M33" s="79" t="s"><v>25</v></c><c r="N33" s="81"/><c r="O33" s="186"/><c r="P33" s="187"/><c r="Q33" s="188"/><c r="R33" s="189"/><c r="S33" s="190"/><c r="T33" s="28"/><c r="U33" s="26"/><c r="W33" s="117" t="e"><f>W30-W27</f><v>#VALUE!</v></c></row><row r="34" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="A34" s="1"/><c r="I34" s="109"><f>I1</f><v>0</v></c><c r="J34" s="136"><f>I9</f><v>0</v></c><c r="L34" s="8"/><c r="M34" s="191" t="s"><v>26</v></c><c r="N34" s="192"/><c r="O34" s="193"/><c r="P34" s="194"/><c r="Q34" s="188"/><c r="R34" s="189"/><c r="S34" s="190"/><c r="T34" s="30"/><c r="U34" s="29"/><c r="V34" s="1"/><c r="W34" s="24"/></row><row r="35" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="A35" s="1"/><c r="D35" s="31"/><c r="I35" s="41"><f>J1</f><v>0</v></c><c r="J35" s="27"><f>J9</f><v>0</v></c><c r="L35"/><c r="M35" s="195" t="s"><v>27</v></c><c r="N35" s="196"/><c r="O35" s="197"/><c r="P35" s="167" t="s"><v>28</v></c><c r="Q35" s="169"/><c r="R35" s="167" t="s"><v>29</v></c><c r="S35" s="169"/><c r="T35" s="167" t="s"><v>30</v></c><c r="U35" s="169"/><c r="V35" s="1"/><c r="W35" s="1"/></row><row r="36" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="B36" s="9"/><c r="I36" s="41"><f>K1</f><v>0</v></c><c r="J36" s="27"><f>K9</f><v>0</v></c><c r="L36"/><c r="M36" s="33" t="s"><v>13</v></c><c r="N36" s="34" t="s"><v>31</v></c><c r="O36" s="35" t="s"><v>32</v></c><c r="P36" s="36" t="s"><v>33</v></c><c r="Q36" s="35" t="s"><v>32</v></c><c r="R36" s="36" t="s"><v>33</v></c><c r="S36" s="35" t="s"><v>32</v></c><c r="T36" s="36" t="s"><v>33</v></c><c r="U36" s="35" t="s"><v>32</v></c><c r="V36" s="1"/><c r="W36" s="1"/></row><row r="37" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="M37" s="37"/><c r="N37" s="38"/><c r="O37" s="39"/><c r="P37" s="151"><v>605655</v></c><c r="Q37" s="77"><v>10000</v></c><c r="R37" s="153"/><c r="S37" s="78"/><c r="T37" s="152"/><c r="U37" s="74"/><c r="A37" s="1"/><c r="I37" s="41"><f>L$1</f><v>0</v></c><c r="J37" s="27"><f>L9</f><v>0</v></c><c r="K37" s="24"/><c r="L37"/><c r="V37" s="1"/><c r="W37" s="18" t="s"><v>14</v></c></row><row r="38"     spans="1:23" x14ac:dyDescent="0.3"><c r="M38" s="37"/><c r="N38" s="38"/><c r="O38" s="39"/><c r="P38" s="152"><v>605656</v></c><c r="Q38" s="66"><v>10001</v></c><c r="R38" s="154"/><c r="S38" s="74"/><c r="T38" s="152"/><c r="U38" s="68"/><c r="A38" s="1"/><c r="I38" s="41"/><c r="J38" s="27"/><c r="K38" s="24"/><c r="L38" s="105"/><c r="V38" s="1"/><c r="W38" s="1" t="s"><v>14</v></c></row><row r="39"     spans="1:23" x14ac:dyDescent="0.3"><c r="M39" s="37"/><c r="N39" s="38"/><c r="O39" s="39"/><c r="P39" s="152"><v>605657</v></c><c r="Q39" s="66"><v>10002</v></c><c r="R39" s="154"/><c r="S39" s="74"/><c r="T39" s="152"/><c r="U39" s="68"/><c r="A39" s="1"/><c r="I39" s="41"/><c r="J39" s="27"/><c r="K39" s="24"/><c r="L39" s="105"/><c r="V39" s="1"/><c r="W39" s="1" t="s"><v>14</v></c></row><row r="40"     spans="1:23" x14ac:dyDescent="0.3"><c r="M40" s="37"/><c r="N40" s="38"/><c r="O40" s="39"/><c r="P40" s="152"><v>605658</v></c><c r="Q40" s="66"><v>10003</v></c><c r="R40" s="154"/><c r="S40" s="74"/><c r="T40" s="152"/><c r="U40" s="68"/><c r="A40" s="1"/><c r="I40" s="41"/><c r="J40" s="27"/><c r="K40" s="24"/><c r="L40" s="105"/><c r="V40" s="1"/><c r="W40" s="1" t="s"><v>14</v></c></row><row r="41"     spans="1:23" x14ac:dyDescent="0.3"><c r="M41" s="37"/><c r="N41" s="38"/><c r="O41" s="39"/><c r="P41" s="152"><v>605659</v></c><c r="Q41" s="66"><v>10004</v></c><c r="R41" s="154"/><c r="S41" s="74"/><c r="T41" s="152"/><c r="U41" s="68"/><c r="A41" s="1"/><c r="I41" s="41"/><c r="J41" s="27"/><c r="K41" s="24"/><c r="L41" s="105"/><c r="V41" s="1"/><c r="W41" s="1" t="s"><v>14</v></c></row><row r="42"     spans="1:23" x14ac:dyDescent="0.3"><c r="M42" s="37"/><c r="N42" s="38"/><c r="O42" s="39"/><c r="P42" s="152"><v>605660</v></c><c r="Q42" s="66"><v>10005</v></c><c r="R42" s="154"/><c r="S42" s="74"/><c r="T42" s="152"/><c r="U42" s="68"/><c r="A42" s="1"/><c r="I42" s="41"/><c r="J42" s="27"/><c r="K42" s="24"/><c r="L42" s="105"/><c r="V42" s="1"/><c r="W42" s="1" t="s"><v>14</v></c></row><row r="43"     spans="1:23" x14ac:dyDescent="0.3"><c r="M43" s="37"/><c r="N43" s="38"/><c r="O43" s="39"/><c r="P43" s="152"><v>605661</v></c><c r="Q43" s="66"><v>10006</v></c><c r="R43" s="154"/><c r="S43" s="74"/><c r="T43" s="152"/><c r="U43" s="68"/><c r="A43" s="1"/><c r="I43" s="41"/><c r="J43" s="27"/><c r="K43" s="24"/><c r="L43" s="105"/><c r="V43" s="1"/><c r="W43" s="1" t="s"><v>14</v></c></row><row r="44"     spans="1:23" x14ac:dyDescent="0.3"><c r="M44" s="37"/><c r="N44" s="38"/><c r="O44" s="39"/><c r="P44" s="152"><v>605662</v></c><c r="Q44" s="66"><v>10007</v></c><c r="R44" s="154"/><c r="S44" s="74"/><c r="T44" s="152"/><c r="U44" s="68"/><c r="A44" s="1"/><c r="I44" s="41"/><c r="J44" s="27"/><c r="K44" s="24"/><c r="L44" s="105"/><c r="V44" s="1"/><c r="W44" s="1" t="s"><v>14</v></c></row><row r="45"     spans="1:23" x14ac:dyDescent="0.3"><c r="M45" s="37"/><c r="N45" s="38"/><c r="O45" s="39"/><c r="P45" s="152"><v>605663</v></c><c r="Q45" s="66"><v>10008</v></c><c r="R45" s="154"/><c r="S45" s="74"/><c r="T45" s="152"/><c r="U45" s="68"/><c r="A45" s="1"/><c r="I45" s="41"/><c r="J45" s="27"/><c r="K45" s="24"/><c r="L45" s="105"/><c r="V45" s="1"/><c r="W45" s="1" t="s"><v>14</v></c></row><row r="46"     spans="1:23" x14ac:dyDescent="0.3"><c r="M46" s="37"/><c r="N46" s="38"/><c r="O46" s="39"/><c r="P46" s="152"><v>605664</v></c><c r="Q46" s="66"><v>10009</v></c><c r="R46" s="154"/><c r="S46" s="74"/><c r="T46" s="152"/><c r="U46" s="68"/><c r="A46" s="1"/><c r="I46" s="41"/><c r="J46" s="27"/><c r="K46" s="24"/><c r="L46" s="105"/><c r="V46" s="1"/><c r="W46" s="1" t="s"><v>14</v></c></row><row r="47"     spans="1:23" x14ac:dyDescent="0.3"><c r="M47" s="37"/><c r="N47" s="38"/><c r="O47" s="39"/><c r="P47" s="152"><v>605665</v></c><c r="Q47" s="66"><v>10010</v></c><c r="R47" s="154"/><c r="S47" s="74"/><c r="T47" s="152"/><c r="U47" s="68"/><c r="A47" s="1"/><c r="I47" s="41"/><c r="J47" s="27"/><c r="K47" s="24"/><c r="L47" s="105"/><c r="V47" s="1"/><c r="W47" s="1" t="s"><v>14</v></c></row><row r="48"     spans="1:23" x14ac:dyDescent="0.3"><c r="M48" s="37"/><c r="N48" s="38"/><c r="O48" s="39"/><c r="P48" s="152"><v>605666</v></c><c r="Q48" s="66"><v>10011</v></c><c r="R48" s="154"/><c r="S48" s="74"/><c r="T48" s="152"/><c r="U48" s="68"/><c r="A48" s="1"/><c r="I48" s="41"/><c r="J48" s="27"/><c r="K48" s="24"/><c r="L48" s="105"/><c r="V48" s="1"/><c r="W48" s="1" t="s"><v>14</v></c></row><row r="49"     spans="1:23" x14ac:dyDescent="0.3"><c r="M49" s="37"/><c r="N49" s="38"/><c r="O49" s="39"/><c r="P49" s="152"><v>605667</v></c><c r="Q49" s="66"><v>10012</v></c><c r="R49" s="154"/><c r="S49" s="74"/><c r="T49" s="152"/><c r="U49" s="68"/><c r="A49" s="1"/><c r="I49" s="41"/><c r="J49" s="27"/><c r="K49" s="24"/><c r="L49" s="105"/><c r="V49" s="1"/><c r="W49" s="1" t="s"><v>14</v></c></row><row r="50"     spans="1:23" x14ac:dyDescent="0.3"><c r="M50" s="37"/><c r="N50" s="38"/><c r="O50" s="39"/><c r="P50" s="152"><v>605668</v></c><c r="Q50" s="66"><v>10013</v></c><c r="R50" s="154"/><c r="S50" s="74"/><c r="T50" s="152"/><c r="U50" s="68"/><c r="A50" s="1"/><c r="I50" s="41"/><c r="J50" s="27"/><c r="K50" s="24"/><c r="L50" s="105"/><c r="V50" s="1"/><c r="W50" s="1" t="s"><v>14</v></c></row><row r="51"     spans="1:23" x14ac:dyDescent="0.3"><c r="M51" s="37"/><c r="N51" s="38"/><c r="O51" s="39"/><c r="P51" s="152"><v>605669</v></c><c r="Q51" s="66"><v>10014</v></c><c r="R51" s="154"/><c r="S51" s="74"/><c r="T51" s="152"/><c r="U51" s="68"/><c r="A51" s="1"/><c r="I51" s="41"/><c r="J51" s="27"/><c r="K51" s="24"/><c r="L51" s="105"/><c r="V51" s="1"/><c r="W51" s="1" t="s"><v>14</v></c></row><row r="52"     spans="1:23" x14ac:dyDescent="0.3"><c r="M52" s="37"/><c r="N52" s="38"/><c r="O52" s="39"/><c r="P52" s="152"><v>605670</v></c><c r="Q52" s="66"><v>10015</v></c><c r="R52" s="154"/><c r="S52" s="74"/><c r="T52" s="152"/><c r="U52" s="68"/><c r="A52" s="1"/><c r="I52" s="41"/><c r="J52" s="27"/><c r="K52" s="24"/><c r="L52" s="105"/><c r="V52" s="1"/><c r="W52" s="1" t="s"><v>14</v></c></row><row r="53"     spans="1:23" x14ac:dyDescent="0.3"><c r="M53" s="37"/><c r="N53" s="38"/><c r="O53" s="39"/><c r="P53" s="152"><v>605671</v></c><c r="Q53" s="66"><v>10016</v></c><c r="R53" s="154"/><c r="S53" s="74"/><c r="T53" s="152"/><c r="U53" s="68"/><c r="A53" s="1"/><c r="I53" s="41"/><c r="J53" s="27"/><c r="K53" s="24"/><c r="L53" s="105"/><c r="V53" s="1"/><c r="W53" s="1" t="s"><v>14</v></c></row><row r="54"     spans="1:23" x14ac:dyDescent="0.3"><c r="M54" s="37"/><c r="N54" s="38"/><c r="O54" s="39"/><c r="P54" s="152"><v>605655</v></c><c r="Q54" s="66"><v>10000</v></c><c r="R54" s="154"/><c r="S54" s="74"/><c r="T54" s="152"/><c r="U54" s="68"/><c r="A54" s="1"/><c r="I54" s="41"/><c r="J54" s="27"/><c r="K54" s="24"/><c r="L54" s="105"/><c r="V54" s="1"/><c r="W54" s="1" t="s"><v>14</v></c></row><row r="55"     spans="1:23" x14ac:dyDescent="0.3"><c r="M55" s="37"/><c r="N55" s="38"/><c r="O55" s="39"/><c r="P55" s="152"><v>605656</v></c><c r="Q55" s="66"><v>10001</v></c><c r="R55" s="154"/><c r="S55" s="74"/><c r="T55" s="152"/><c r="U55" s="68"/><c r="A55" s="1"/><c r="I55" s="41"/><c r="J55" s="27"/><c r="K55" s="24"/><c r="L55" s="105"/><c r="V55" s="1"/><c r="W55" s="1" t="s"><v>14</v></c></row><row r="56"     spans="1:23" x14ac:dyDescent="0.3"><c r="M56" s="37"/><c r="N56" s="38"/><c r="O56" s="39"/><c r="P56" s="152"><v>605657</v></c><c r="Q56" s="66"><v>10002</v></c><c r="R56" s="154"/><c r="S56" s="74"/><c r="T56" s="152"/><c r="U56" s="68"/><c r="A56" s="1"/><c r="I56" s="41"/><c r="J56" s="27"/><c r="K56" s="24"/><c r="L56" s="105"/><c r="V56" s="1"/><c r="W56" s="1" t="s"><v>14</v></c></row><row r="57"     spans="1:23" x14ac:dyDescent="0.3"><c r="M57" s="37"/><c r="N57" s="38"/><c r="O57" s="39"/><c r="P57" s="152"><v>605658</v></c><c r="Q57" s="66"><v>10003</v></c><c r="R57" s="154"/><c r="S57" s="74"/><c r="T57" s="152"/><c r="U57" s="68"/><c r="A57" s="1"/><c r="I57" s="41"/><c r="J57" s="27"/><c r="K57" s="24"/><c r="L57" s="105"/><c r="V57" s="1"/><c r="W57" s="1" t="s"><v>14</v></c></row><row r="58"     spans="1:23" x14ac:dyDescent="0.3"><c r="M58" s="37"/><c r="N58" s="38"/><c r="O58" s="39"/><c r="P58" s="152"><v>605659</v></c><c r="Q58" s="66"><v>10004</v></c><c r="R58" s="154"/><c r="S58" s="74"/><c r="T58" s="152"/><c r="U58" s="68"/><c r="A58" s="1"/><c r="I58" s="41"/><c r="J58" s="27"/><c r="K58" s="24"/><c r="L58" s="105"/><c r="V58" s="1"/><c r="W58" s="1" t="s"><v>14</v></c></row><row r="59"     spans="1:23" x14ac:dyDescent="0.3"><c r="M59" s="37"/><c r="N59" s="38"/><c r="O59" s="39"/><c r="P59" s="152"><v>605660</v></c><c r="Q59" s="66"><v>10005</v></c><c r="R59" s="154"/><c r="S59" s="74"/><c r="T59" s="152"/><c r="U59" s="68"/><c r="A59" s="1"/><c r="I59" s="41"/><c r="J59" s="27"/><c r="K59" s="24"/><c r="L59" s="105"/><c r="V59" s="1"/><c r="W59" s="1" t="s"><v>14</v></c></row><row r="60"     spans="1:23" x14ac:dyDescent="0.3"><c r="M60" s="37"/><c r="N60" s="38"/><c r="O60" s="39"/><c r="P60" s="152"><v>605661</v></c><c r="Q60" s="66"><v>10006</v></c><c r="R60" s="154"/><c r="S60" s="74"/><c r="T60" s="152"/><c r="U60" s="68"/><c r="A60" s="1"/><c r="I60" s="41"/><c r="J60" s="27"/><c r="K60" s="24"/><c r="L60" s="105"/><c r="V60" s="1"/><c r="W60" s="1" t="s"><v>14</v></c></row><row r="61"     spans="1:23" x14ac:dyDescent="0.3"><c r="M61" s="37"/><c r="N61" s="38"/><c r="O61" s="39"/><c r="P61" s="152"><v>605662</v></c><c r="Q61" s="66"><v>10007</v></c><c r="R61" s="154"/><c r="S61" s="74"/><c r="T61" s="152"/><c r="U61" s="68"/><c r="A61" s="1"/><c r="I61" s="41"/><c r="J61" s="27"/><c r="K61" s="24"/><c r="L61" s="105"/><c r="V61" s="1"/><c r="W61" s="1" t="s"><v>14</v></c></row><row r="62"     spans="1:23" x14ac:dyDescent="0.3"><c r="M62" s="37"/><c r="N62" s="38"/><c r="O62" s="39"/><c r="P62" s="152"><v>605663</v></c><c r="Q62" s="66"><v>10008</v></c><c r="R62" s="154"/><c r="S62" s="74"/><c r="T62" s="152"/><c r="U62" s="68"/><c r="A62" s="1"/><c r="I62" s="41"/><c r="J62" s="27"/><c r="K62" s="24"/><c r="L62" s="105"/><c r="V62" s="1"/><c r="W62" s="1" t="s"><v>14</v></c></row><row r="63"     spans="1:23" x14ac:dyDescent="0.3"><c r="M63" s="37"/><c r="N63" s="38"/><c r="O63" s="39"/><c r="P63" s="152"><v>605664</v></c><c r="Q63" s="66"><v>10009</v></c><c r="R63" s="154"/><c r="S63" s="74"/><c r="T63" s="152"/><c r="U63" s="68"/><c r="A63" s="1"/><c r="I63" s="41"/><c r="J63" s="27"/><c r="K63" s="24"/><c r="L63" s="105"/><c r="V63" s="1"/><c r="W63" s="1" t="s"><v>14</v></c></row><row r="64"     spans="1:23" x14ac:dyDescent="0.3"><c r="M64" s="37"/><c r="N64" s="38"/><c r="O64" s="39"/><c r="P64" s="152"><v>605665</v></c><c r="Q64" s="66"><v>10010</v></c><c r="R64" s="154"/><c r="S64" s="74"/><c r="T64" s="152"/><c r="U64" s="68"/><c r="A64" s="1"/><c r="I64" s="41"/><c r="J64" s="27"/><c r="K64" s="24"/><c r="L64" s="105"/><c r="V64" s="1"/><c r="W64" s="1" t="s"><v>14</v></c></row><row r="65"     spans="1:23" x14ac:dyDescent="0.3"><c r="M65" s="37"/><c r="N65" s="38"/><c r="O65" s="39"/><c r="P65" s="152"><v>605666</v></c><c r="Q65" s="66"><v>10011</v></c><c r="R65" s="154"/><c r="S65" s="74"/><c r="T65" s="152"/><c r="U65" s="68"/><c r="A65" s="1"/><c r="I65" s="41"/><c r="J65" s="27"/><c r="K65" s="24"/><c r="L65" s="105"/><c r="V65" s="1"/><c r="W65" s="1" t="s"><v>14</v></c></row><row r="66"     spans="1:23" x14ac:dyDescent="0.3"><c r="M66" s="37"/><c r="N66" s="38"/><c r="O66" s="39"/><c r="P66" s="152"><v>605667</v></c><c r="Q66" s="66"><v>10012</v></c><c r="R66" s="154"/><c r="S66" s="74"/><c r="T66" s="152"/><c r="U66" s="68"/><c r="A66" s="1"/><c r="I66" s="41"/><c r="J66" s="27"/><c r="K66" s="24"/><c r="L66" s="105"/><c r="V66" s="1"/><c r="W66" s="1" t="s"><v>14</v></c></row><row r="67"     spans="1:23" x14ac:dyDescent="0.3"><c r="M67" s="37"/><c r="N67" s="38"/><c r="O67" s="39"/><c r="P67" s="152"><v>605668</v></c><c r="Q67" s="66"><v>10013</v></c><c r="R67" s="154"/><c r="S67" s="74"/><c r="T67" s="152"/><c r="U67" s="68"/><c r="A67" s="1"/><c r="I67" s="41"/><c r="J67" s="27"/><c r="K67" s="24"/><c r="L67" s="105"/><c r="V67" s="1"/><c r="W67" s="1" t="s"><v>14</v></c></row><row r="68"     spans="1:23" x14ac:dyDescent="0.3"><c r="M68" s="37"/><c r="N68" s="38"/><c r="O68" s="39"/><c r="P68" s="152"><v>605669</v></c><c r="Q68" s="66"><v>10014</v></c><c r="R68" s="154"/><c r="S68" s="74"/><c r="T68" s="152"/><c r="U68" s="68"/><c r="A68" s="1"/><c r="I68" s="41"/><c r="J68" s="27"/><c r="K68" s="24"/><c r="L68" s="105"/><c r="V68" s="1"/><c r="W68" s="1" t="s"><v>14</v></c></row><row r="69"     spans="1:23" x14ac:dyDescent="0.3"><c r="M69" s="37"/><c r="N69" s="38"/><c r="O69" s="39"/><c r="P69" s="152"><v>605670</v></c><c r="Q69" s="66"><v>10015</v></c><c r="R69" s="154"/><c r="S69" s="74"/><c r="T69" s="152"/><c r="U69" s="68"/><c r="A69" s="1"/><c r="I69" s="41"/><c r="J69" s="27"/><c r="K69" s="24"/><c r="L69" s="105"/><c r="V69" s="1"/><c r="W69" s="1" t="s"><v>14</v></c></row><row r="70"     spans="1:23" x14ac:dyDescent="0.3"><c r="M70" s="37"/><c r="N70" s="38"/><c r="O70" s="39"/><c r="P70" s="152"><v>605671</v></c><c r="Q70" s="66"><v>10016</v></c><c r="R70" s="154"/><c r="S70" s="74"/><c r="T70" s="152"/><c r="U70" s="68"/><c r="A70" s="1"/><c r="I70" s="41"/><c r="J70" s="27"/><c r="K70" s="24"/><c r="L70" s="105"/><c r="V70" s="1"/><c r="W70" s="1" t="s"><v>14</v></c></row><row r="71" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="B71" s="20"/><c r="C71" s="32"/><c r="I71" s="41"><f t="shared" ref="I71:I78" si="6">L$1</f><v>0</v></c><c r="J71" s="27"><f t="shared" ref="J71:J78" si="7">L10</f><v>0</v></c><c r="L71" s="105"/><c r="M71" s="171" t="s"><v>42</v></c><c r="N71" s="179"/><c r="O71" s="150"/><c r="P71" s="152"/><c r="Q71" s="75"/><c r="R71" s="154"/><c r="S71" s="73"/><c r="T71" s="152"/><c r="U71" s="76"/><c r="V71" s="1"/><c r="W71" s="1"/></row><row r="72" spans="1:23" x14ac:dyDescent="0.3"><c r="M72" s="37" t="inlineStr"><is><t xml:space="preserve">30-07-2026</t></is></c><c r="N72" s="38" t="inlineStr"><is><t xml:space="preserve">BCI</t></is></c><c r="O72" s="39"><v>127092</v></c><c r="B72" s="20"/><c r="C72" s="32"/><c r="I72" s="41"><f t="shared" si="6"/></row><row r="73" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.4"><c r="M73" s="37" t="inlineStr"><is><t xml:space="preserve">30-07-2026</t></is></c><c r="N73" s="38" t="inlineStr"><is><t xml:space="preserve">BCI</t></is></c><c r="O73" s="39"><v>972618</v></c></row><row r="74" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3"><c r="M74" s="37" t="inlineStr"><is><t xml:space="preserve">30-07-2026</t></is></c><c r="N74" s="38" t="inlineStr"><is><t xml:space="preserve">BCI</t></is></c><c r="O74" s="39"><v>368449</v></c></row><row r="75" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.6"><c r="M75" s="37" t="inlineStr"><is><t xml:space="preserve">30-07-2026</t></is></c><c r="N75" s="38" t="inlineStr"><is><t xml:space="preserve">BCI</t></is></c><c r="O75" s="39"><v>92552</v></c></row><row r="76" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.6"></row><row r="77" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3"></row><row r="78" spans="1:23" x14ac:dyDescent="0.3"></row><row r="79" spans="1:23" x14ac:dyDescent="0.3"><c r="L79" s="105"/><c r="M79" s="37"/><c r="N79" s="38"/><c r="O79" s="39"/><c r="P79" s="152"/><c r="Q79" s="66"/><c r="R79" s="152"/><c r="S79" s="67"/><c r="T79" s="152"/><c r="U79" s="68"/></row><row r="80" spans="1:23" x14ac:dyDescent="0.3"><c r="A80" s="20"/><c r="B80" s="20"/><c r="C80" s="40"/><c r="D80" s="170"/><c r="E80" s="170"/><c r="F80" s="17"/><c r="G80" s="1"/><c r="H80" s="64"/><c r="I80" s="13"/><c r="J80" s="53"/><c r="K80" s="24"/><c r="L80" s="105"/><c r="M80" s="37"/><c r="N80" s="38"/><c r="O80" s="39"/><c r="P80" s="152"/><c r="Q80" s="66"/><c r="R80" s="152"/><c r="S80" s="67"/><c r="T80" s="152"/><c r="U80" s="68"/></row><row r="81" spans="1:23" x14ac:dyDescent="0.3"><c r="A81" s="20"/><c r="B81" s="20"/><c r="C81" s="40"/><c r="D81" s="170"/><c r="E81" s="170"/><c r="F81" s="23"/><c r="G81" s="1"/><c r="H81" s="64"/><c r="I81" s="13"/><c r="J81" s="53"/><c r="L81" s="105"/><c r="M81" s="37"/><c r="N81" s="38"/><c r="O81" s="39"/><c r="P81" s="152"/><c r="Q81" s="66"/><c r="R81" s="152"/><c r="S81" s="67"/><c r="T81" s="154"/><c r="U81" s="68"/></row><row r="82" spans="1:21" x14ac:dyDescent="0.3"><c r="A82" s="20"/><c r="B82" s="20"/><c r="C82" s="40"/><c r="D82" s="170"/><c r="E82" s="170"/><c r="F82" s="23"/><c r="G82" s="1"/><c r="H82" s="46"/><c r="I82" s="13"/><c r="J82" s="53"/><c r="L82" s="105"/><c r="M82" s="37"/><c r="N82" s="38"/><c r="O82" s="39"/><c r="P82" s="152"/><c r="Q82" s="66"/><c r="R82" s="152"/><c r="S82" s="67"/><c r="T82" s="154"/><c r="U82" s="68"/></row><row r="83" spans="1:21" x14ac:dyDescent="0.3"><c r="A83" s="20"/><c r="B83" s="20"/><c r="C83" s="40"/><c r="D83" s="23"/><c r="E83" s="25"/><c r="F83" s="23"/><c r="G83" s="1"/><c r="H83" s="46"/><c r="I83" s="13"/><c r="J83" s="53"/><c r="L83" s="105"/><c r="M83" s="37"/><c r="N83" s="38"/><c r="O83" s="39"/><c r="P83" s="152"/><c r="Q83" s="66"/><c r="R83" s="152"/><c r="S83" s="67"/><c r="T83" s="154"/><c r="U83" s="68"/></row><row r="84" spans="1:21" x14ac:dyDescent="0.3"><c r="A84" s="20"/><c r="B84" s="20"/><c r="C84" s="40"/><c r="D84" s="185"/><c r="E84" s="185"/><c r="F84" s="23"/><c r="G84" s="1"/><c r="H84" s="46"/><c r="I84" s="13"/><c r="J84" s="53"/><c r="L84" s="105"/><c r="M84" s="37"/><c r="N84" s="38"/><c r="O84" s="39"/><c r="P84" s="151"/><c r="Q84" s="66"/><c r="R84" s="152"/><c r="S84" s="67"/><c r="T84" s="154"/><c r="U84" s="68"/></row><row r="85" spans="1:21" x14ac:dyDescent="0.3"><c r="A85" s="20"/><c r="B85" s="51"/><c r="C85" s="40"/><c r="D85" s="178"/><c r="E85" s="178"/><c r="F85" s="23"/><c r="G85" s="1"/><c r="H85" s="46"/><c r="I85" s="50"/><c r="J85" s="53"/><c r="L85" s="105"/><c r="M85" s="37"/><c r="N85" s="38"/><c r="O85" s="39"/><c r="P85" s="151"/><c r="Q85" s="66"/><c r="R85" s="152"/><c r="S85" s="67"/><c r="T85" s="154"/><c r="U85" s="68"/></row><row r="86" spans="1:21" x14ac:dyDescent="0.3"><c r="A86" s="25"/><c r="B86" s="51"/><c r="C86" s="40"/><c r="D86" s="166"/><c r="E86" s="166"/><c r="F86" s="23"/><c r="G86" s="1"/><c r="H86" s="46"/><c r="I86" s="50"/><c r="J86" s="53"/><c r="L86" s="18"/><c r="M86" s="37"/><c r="N86" s="38"/><c r="O86" s="39"/><c r="P86" s="152"/><c r="Q86" s="66"/><c r="R86" s="152"/><c r="S86" s="67"/><c r="T86" s="154"/><c r="U86" s="68"/></row><row r="87" spans="1:21" x14ac:dyDescent="0.3"><c r="A87" s="20"/><c r="B87" s="51"/><c r="C87" s="40"/><c r="D87" s="166"/><c r="E87" s="166"/><c r="F87" s="23"/><c r="G87" s="1"/><c r="H87" s="46"/><c r="I87" s="50"/><c r="J87" s="53"/><c r="L87" s="18"/><c r="M87" s="37"/><c r="N87" s="38"/><c r="O87" s="39"/><c r="P87" s="152"/><c r="Q87" s="66"/><c r="R87" s="152"/><c r="S87" s="67"/><c r="T87" s="154"/><c r="U87" s="68"/></row><row r="88" spans="1:21" x14ac:dyDescent="0.3"><c r="A88" s="20"/><c r="B88" s="51"/><c r="C88" s="40"/><c r="D88" s="22"/><c r="E88" s="22"/><c r="F88" s="23"/><c r="G88" s="1"/><c r="H88" s="46"/><c r="I88" s="50"/><c r="J88" s="53"/><c r="L88" s="18"/><c r="M88" s="37"/><c r="N88" s="38"/><c r="O88" s="39"/><c r="P88" s="152"/><c r="Q88" s="66"/><c r="R88" s="152"/><c r="S88" s="67"/><c r="T88" s="154"/><c r="U88" s="68"/></row><row r="89" spans="1:21" x14ac:dyDescent="0.3"><c r="A89" s="20"/><c r="B89"/><c r="C89" s="40"/><c r="D89" s="22"/><c r="E89" s="22"/><c r="F89" s="23"/><c r="G89" s="1"/><c r="H89" s="46"/><c r="I89" s="50"/><c r="J89" s="53"/><c r="L89" s="18"/><c r="M89" s="37"/><c r="N89" s="38"/><c r="O89" s="39"/><c r="P89" s="152"/><c r="Q89" s="66"/><c r="R89" s="152"/><c r="S89" s="67"/><c r="T89" s="154"/><c r="U89" s="68"/></row><row r="90" spans="1:21" x14ac:dyDescent="0.3"><c r="A90" s="20"/><c r="B90"/><c r="C90" s="40"/><c r="D90" s="22"/><c r="E90" s="22"/><c r="F90" s="23"/><c r="G90" s="1"/><c r="H90" s="46"/><c r="I90" s="50"/><c r="J90" s="53"/><c r="L90" s="18"/><c r="M90" s="37"/><c r="N90" s="38"/><c r="O90" s="39"/><c r="P90" s="152"/><c r="Q90" s="66"/><c r="R90" s="152"/><c r="S90" s="67"/><c r="T90" s="154"/><c r="U90" s="68"/></row><row r="91" spans="1:21" x14ac:dyDescent="0.3"><c r="A91" s="20"/><c r="B91"/><c r="C91" s="40"/><c r="D91" s="22"/><c r="E91" s="22"/><c r="F91" s="23"/><c r="G91" s="1"/><c r="H91" s="46"/><c r="I91" s="50"/><c r="J91" s="53"/><c r="L91" s="18"/><c r="M91" s="37"/><c r="N91" s="38"/><c r="O91" s="39"/><c r="P91" s="152"/><c r="Q91" s="66"/><c r="R91" s="152"/><c r="S91" s="67"/><c r="T91" s="154"/><c r="U91" s="68"/></row><row r="92" spans="1:21" x14ac:dyDescent="0.3"><c r="A92" s="20"/><c r="B92"/><c r="C92" s="40"/><c r="D92" s="22"/><c r="E92" s="22"/><c r="F92" s="23"/><c r="G92" s="1"/><c r="H92" s="46"/><c r="I92" s="50"/><c r="J92" s="53"/><c r="L92" s="18"/><c r="M92" s="37"/><c r="N92" s="38"/><c r="O92" s="39"/><c r="P92" s="152"/><c r="Q92" s="66"/><c r="R92" s="152"/><c r="S92" s="67"/><c r="T92" s="154"/><c r="U92" s="68"/></row><row r="93" spans="1:21" x14ac:dyDescent="0.3"><c r="A93" s="25"/><c r="B93"/><c r="C93" s="40"/><c r="D93" s="166"/><c r="E93" s="166"/><c r="F93" s="23"/><c r="G93" s="1"/><c r="H93" s="46"/><c r="I93" s="50"/><c r="J93" s="53"/><c r="L93" s="18"/><c r="M93" s="37"/><c r="N93" s="38"/><c r="O93" s="39"/><c r="P93" s="152"/><c r="Q93" s="66"/><c r="R93" s="152"/><c r="S93" s="67"/><c r="T93" s="154"/><c r="U93" s="68"/></row><row r="94" spans="1:21" x14ac:dyDescent="0.3"><c r="A94" s="25"/><c r="B94"/><c r="C94" s="40"/><c r="D94" s="22"/><c r="E94" s="22"/><c r="F94" s="23"/><c r="G94" s="1"/><c r="H94" s="46"/><c r="I94" s="50"/><c r="J94" s="53"/><c r="L94" s="18"/><c r="M94" s="37"/><c r="N94" s="38"/><c r="O94" s="39"/><c r="P94" s="152"/><c r="Q94" s="135"/><c r="R94" s="155"/><c r="S94" s="88"/><c r="T94" s="154"/><c r="U94" s="68"/></row><row r="95" spans="1:21" x14ac:dyDescent="0.3"><c r="A95" s="25"/><c r="B95"/><c r="C95" s="40"/><c r="D95" s="22"/><c r="E95" s="22"/><c r="F95" s="23"/><c r="G95" s="1"/><c r="H95" s="46"/><c r="I95" s="50"/><c r="J95" s="53"/><c r="L95" s="18"/><c r="M95" s="37"/><c r="N95" s="38"/><c r="O95" s="39"/><c r="P95" s="152"/><c r="Q95" s="135"/><c r="R95" s="155"/><c r="S95" s="88"/><c r="T95" s="154"/><c r="U95" s="68"/></row><row r="96" spans="1:21" x14ac:dyDescent="0.3"><c r="A96" s="25"/><c r="B96"/><c r="C96" s="40"/><c r="D96" s="22"/><c r="E96" s="22"/><c r="F96" s="23"/><c r="G96" s="1"/><c r="H96" s="46"/><c r="I96" s="50"/><c r="J96" s="53"/><c r="L96" s="18"/><c r="M96" s="37"/><c r="N96" s="38"/><c r="O96" s="39"/><c r="P96" s="152"/><c r="Q96" s="135"/><c r="R96" s="155"/><c r="S96" s="88"/><c r="T96" s="154"/><c r="U96" s="68"/></row><row r="97" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="A97" s="25"/><c r="B97"/><c r="C97" s="40"/><c r="D97" s="166"/><c r="E97" s="166"/><c r="F97" s="23"/><c r="G97" s="1"/><c r="H97" s="46"/><c r="I97" s="50"/><c r="J97" s="53"/><c r="L97" s="18"/><c r="M97" s="37"/><c r="N97" s="38"/><c r="O97" s="39"/><c r="P97" s="152"/><c r="Q97" s="84"/><c r="R97" s="155"/><c r="S97" s="88"/><c r="T97" s="154"/><c r="U97" s="71"/></row><row r="98" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"><c r="A98" s="25"/><c r="B98"/><c r="C98" s="40"/><c r="D98" s="166"/><c r="E98" s="166"/><c r="F98" s="20"/><c r="G98" s="1"/><c r="H98" s="46"/><c r="I98" s="50"/><c r="J98" s="53"/><c r="L98"/><c r="M98" s="171" t="s"><v>34</v></c><c r="N98" s="172"/><c r="O98" s="42"><v>1560711</v></c><c r="P98" s="52" t="s"><v>11</v></c><c r="Q98" s="42"/><c r="R98" s="52" t="s"><v>11</v></c><c r="S98" s="42"/><c r="T98" s="52" t="s"><v>11</v></c><c r="U98" s="42"/></row><row r="99" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="A99" s="25"/><c r="B99"/><c r="C99" s="90"/><c r="D99" s="166"/><c r="E99" s="166"/><c r="F99" s="23"/><c r="G99" s="1"/><c r="H99" s="46"/><c r="I99" s="50"/><c r="J99"/><c r="L99"/><c r="M99" s="54"/><c r="N99" s="55"/><c r="O99" s="70"/><c r="P99" s="23"/><c r="Q99" s="69"/><c r="R99" s="70"/><c r="S99" s="70"/><c r="T99" s="6"/></row><row r="100" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"><c r="A100" s="25"/><c r="B100"/><c r="C100" s="25"/><c r="D100" s="22"/><c r="E100" s="22"/><c r="F100" s="23"/><c r="G100" s="1"/><c r="H100" s="46"/><c r="I100" s="50"/><c r="J100"/><c r="L100"/><c r="M100" s="167" t="s"><v>47</v></c><c r="N100" s="168"/><c r="O100" s="169"/><c r="P100" s="181"/><c r="Q100" s="182"/><c r="R100" s="167" t="s"><v>37</v></c><c r="S100" s="168"/><c r="T100" s="183" t="str"><f>Q25</f></c><c r="U100" s="184"/></row><row r="101" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"><c r="A101" s="25"/><c r="B101"/><c r="C101" s="25"/><c r="D101" s="166"/><c r="E101" s="166"/><c r="F101" s="63"/><c r="G101" s="1"/><c r="H101" s="46"/><c r="I101" s="50"/><c r="J101"/><c r="L101"/><c r="M101" s="56"/><c r="N101" s="83"/><c r="O101" s="83"/><c r="P101" s="57"/><c r="Q101" s="58"/><c r="R101" s="58"/><c r="S101" s="58"/><c r="T101" s="56"/><c r="U101" s="56"/></row><row r="102" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"><c r="A102" s="25"/><c r="B102" s="90"/><c r="C102" s="25"/><c r="D102" s="166"/><c r="E102" s="166"/><c r="F102" s="63"/><c r="G102" s="1"/><c r="H102" s="46"/><c r="I102" s="50"/><c r="J102"/><c r="L102"/><c r="M102" s="171" t="s"><v>35</v></c><c r="N102" s="179"/><c r="O102" s="179"/><c r="P102" s="179"/><c r="Q102" s="179"/><c r="R102" s="179"/><c r="S102" s="179"/><c r="T102" s="179"/><c r="U102" s="180"/><c r="V102" s="51"/></row><row r="103" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35"><c r="A103" s="25"/><c r="B103" s="20"/><c r="C103" s="25"/><c r="D103" s="166"/><c r="E103" s="166"/><c r="F103" s="63"/><c r="G103" s="1"/><c r="H103" s="46"/><c r="I103" s="50"/><c r="J103"/><c r="L103" s="49" t="s"><v>59</v></c><c r="M103" s="130" t="s"><v>55</v></c><c r="N103" s="131"/><c r="O103" s="131"/><c r="P103" s="131" t="s"><v>56</v></c><c r="Q103" s="131"/><c r="R103" s="131"/><c r="S103" s="131"/><c r="T103" s="131" t="s"><v>57</v></c><c r="U103" s="132" t="s"><v>60</v></c><c r="V103" s="144" t="s"><v>58</v></c><c r="W103" s="144" t="s"><v>50</v></c></row><row r="104" spans="1:23" ht="15.6" x14ac:dyDescent="0.3"><c r="L104" s="0"/><c r="M104" s="59"/><c r="P104" s="62"/><c r="T104" s="133"/><c r="V104" s="51"/><c r="R104" s="177" t="inlineStr"><is><t xml:space="preserve">CREDITO</t></is></c><c r="A104" s="25"/><c r="B104" s="115"/><c r="C104" s="25"/><c r="D104" s="166"/><c r="E104" s="166"/><c r="F104" s="63"/><c r="G104" s="1"/><c r="H104" s="46"/><c r="I104" s="50"/><c r="J104" s="23"/><c r="N104" s="60"/><c r="O104" s="143" t="s"><v>43</v></c><c r="Q104" s="61"/><c r="S104" s="177"/><c r="U104" s="134"/></row><row r="105" spans="1:23" ht="15.6" x14ac:dyDescent="0.3"><c r="B105" s="51"/><c r="C105" s="89"/><c r="D105" s="166"/><c r="E105" s="166"/><c r="F105" s="63"/><c r="I105" s="115"/><c r="L105"/><c r="M105" s="85"/><c r="N105" s="86"/><c r="O105" s="18"/><c r="P105" s="87"/><c r="Q105" s="56"/><c r="R105" s="175"/><c r="S105" s="175"/><c r="T105" s="65"/><c r="U105" s="95"/><c r="V105" s="51"/></row><row r="106" spans="1:23" ht="15.6" x14ac:dyDescent="0.3"><c r="L106" s="45"/><c r="M106" s="85"/><c r="P106" s="87"/><c r="T106" s="65"/><c r="U106" s="95"/><c r="R106" s="175" t="inlineStr"><is><t xml:space="preserve">TRANSFERENCIA</t></is></c><c r="A106" s="49"/><c r="B106" s="89"/><c r="C106" s="89"/><c r="D106" s="23"/><c r="E106" s="25"/><c r="F106" s="63"/><c r="I106" s="115"/><c r="N106" s="86"/><c r="O106" s="18" t="s"><v>43</v></c><c r="Q106" s="56"/><c r="S106" s="175"/><c r="V106" s="51"/></row><row r="107" spans="1:23" ht="15.6" x14ac:dyDescent="0.3"><c r="L107" s="45"/><c r="M107" s="85"/><c r="N107" s="86"/><c r="O107" s="123"/><c r="P107" s="87"/><c r="Q107" s="56"/><c r="R107" s="175"/><c r="S107" s="175"/><c r="T107" s="65"/><c r="U107" s="95"/><c r="V107" s="51"/></row><row r="108" spans="1:23" ht="15.6" x14ac:dyDescent="0.3"><c r="L108" s="45"/><c r="M108" s="137" t="s"><v>61</v></c><c r="N108" s="138"/><c r="O108" s="139"/><c r="P108" s="140"/><c r="Q108" s="141"/><c r="R108" s="176"/><c r="S108" s="176"/><c r="T108" s="173"/><c r="U108" s="174"/><c r="V108" s="51"/></row><row r="109" spans="1:23" ht="15.6" x14ac:dyDescent="0.3"><c r="L109" s="45"/><c r="M109" s="137" t="s"><v>62</v></c><c r="N109" s="138"/><c r="O109" s="139"/><c r="P109" s="140"/><c r="Q109" s="141"/><c r="R109" s="142"/><c r="S109" s="142"/><c r="T109" s="173"/><c r="U109" s="174"/><c r="V109" s="51"/></row><row r="110" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"><c r="L110" s="45"/><c r="M110" s="94"/><c r="N110" s="64"/><c r="O110" s="123"/><c r="P110" s="87"/><c r="Q110" s="56"/><c r="R110" s="56"/><c r="S110" s="56"/><c r="T110" s="65"/><c r="U110" s="95"/><c r="V110" s="51"/></row><row r="111" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"><c r="L111" s="45"/><c r="M111" s="101" t="s"><v>11</v></c><c r="N111" s="102"><f>SUM(N109:N110)</f><v>0</v></c><c r="O111" s="96"/><c r="P111" s="98"/><c r="Q111" s="97"/><c r="R111" s="97"/><c r="S111" s="97"/><c r="T111" s="99"/><c r="U111" s="100"/><c r="V111" s="51"/></row><row r="112" spans="1:23" x14ac:dyDescent="0.3"><c r="M112"/><c r="O112" s="5"/><c r="Q112"/><c r="S112"/><c r="T112" s="6"/><c r="V112" s="51"/></row><row r="113" spans="1:23" x14ac:dyDescent="0.3"><c r="O113"/><c r="V113" s="51"/></row><row r="114" spans="13:22" x14ac:dyDescent="0.3"><c r="M114" s="23"/><c r="N114" s="23"/><c r="O114" s="23"/><c r="P114" s="23"/><c r="Q114" s="23"/><c r="V114" s="51"/></row><row r="115" spans="13:22" x14ac:dyDescent="0.3"><c r="V115" s="51"/></row><row r="116" spans="13:22" x14ac:dyDescent="0.3"><c r="V116" s="51"/></row><row r="117" spans="13:22" x14ac:dyDescent="0.3"><c r="V117" s="51"/></row><row r="118" spans="13:22" x14ac:dyDescent="0.3"><c r="V118" s="51"/></row><row r="119" spans="13:22" x14ac:dyDescent="0.3"><c r="V119" s="51"/></row><row r="120" spans="13:22" x14ac:dyDescent="0.3"><c r="V120" s="51"/></row><row r="121" spans="13:22" x14ac:dyDescent="0.3"><c r="V121" s="51"/></row><row r="122" spans="13:22" x14ac:dyDescent="0.3"><c r="V122" s="51"/></row><row r="123" spans="13:22" x14ac:dyDescent="0.3"><c r="V123" s="51"/></row><row r="124" spans="13:22" x14ac:dyDescent="0.3"><c r="V124" s="51"/></row><row r="125" spans="13:22" x14ac:dyDescent="0.3"><c r="V125" s="51"/></row><row r="126" spans="13:22" x14ac:dyDescent="0.3"><c r="V126" s="51"/></row><row r="127" spans="13:22" x14ac:dyDescent="0.3"><c r="V127" s="51"/></row><row r="128" spans="13:22" x14ac:dyDescent="0.3"><c r="V128" s="51"/></row><row r="129" spans="13:22" x14ac:dyDescent="0.3"><c r="V129" s="51"/></row><row r="130" spans="22:22" x14ac:dyDescent="0.3"><c r="V130" s="51"/></row><row r="131" spans="22:22" x14ac:dyDescent="0.3"><c r="V131" s="51"/></row><row r="132" spans="22:22" x14ac:dyDescent="0.3"><c r="V132" s="51"/></row><row r="133" spans="22:22" x14ac:dyDescent="0.3"><c r="V133" s="51"/></row><row r="134" spans="22:22" x14ac:dyDescent="0.3"><c r="V134" s="51"/></row><row r="135" spans="22:22" x14ac:dyDescent="0.3"><c r="V135" s="51"/></row><row r="136" spans="22:22" x14ac:dyDescent="0.3"><c r="V136" s="51"/></row><row r="137" spans="22:22" x14ac:dyDescent="0.3"><c r="V137" s="51"/></row><row r="138" spans="22:22" x14ac:dyDescent="0.3"><c r="V138" s="51"/></row><row r="139" spans="22:22" x14ac:dyDescent="0.3"><c r="V139" s="51"/></row><row r="140" spans="22:22" x14ac:dyDescent="0.3"><c r="V140" s="51"/></row><row r="141" spans="22:22" x14ac:dyDescent="0.3"><c r="V141" s="51"/></row><row r="142" spans="22:22" x14ac:dyDescent="0.3"><c r="V142" s="51"/></row><row r="143" spans="22:22" x14ac:dyDescent="0.3"><c r="V143" s="51"/></row><row r="144" spans="22:22" x14ac:dyDescent="0.3"><c r="V144" s="51"/></row><row r="145" spans="22:22" x14ac:dyDescent="0.3"><c r="V145" s="51"/></row></sheetData><mergeCells count="70"><mergeCell ref="M25:N25"/><mergeCell ref="O30:P30"/><mergeCell ref="Q30:S30"/><mergeCell ref="T30:U30"/><mergeCell ref="Q32:S32"/><mergeCell ref="M31:N31"/><mergeCell ref="O31:P31"/><mergeCell ref="Q31:S31"/><mergeCell ref="M30:N30"/><mergeCell ref="M32:N32"/><mergeCell ref="O32:P32"/><mergeCell ref="M22:U22"/><mergeCell ref="Q26:S26"/><mergeCell ref="O29:P29"/><mergeCell ref="Q29:S29"/><mergeCell ref="T29:U29"/><mergeCell ref="T28:U28"/><mergeCell ref="O28:P28"/><mergeCell ref="Q28:S28"/><mergeCell ref="M28:N28"/><mergeCell ref="M29:N29"/><mergeCell ref="O27:P27"/><mergeCell ref="Q27:S27"/><mergeCell ref="T27:U27"/><mergeCell ref="N23:S23"/><mergeCell ref="N24:S24"/><mergeCell ref="T25:U25"/><mergeCell ref="D76:E76"/><mergeCell ref="R35:S35"/><mergeCell ref="T35:U35"/><mergeCell ref="O33:P33"/><mergeCell ref="Q33:S33"/><mergeCell ref="M34:N34"/><mergeCell ref="O34:P34"/><mergeCell ref="Q34:S34"/><mergeCell ref="P35:Q35"/><mergeCell ref="M35:O35"/><mergeCell ref="M71:N71"/><mergeCell ref="D104:E104"/><mergeCell ref="D105:E105"/><mergeCell ref="D85:E85"/><mergeCell ref="M102:U102"/><mergeCell ref="R100:S100"/><mergeCell ref="D101:E101"/><mergeCell ref="P100:Q100"/><mergeCell ref="T100:U100"/><mergeCell ref="D93:E93"/><mergeCell ref="D99:E99"/><mergeCell ref="D86:E86"/><mergeCell ref="D98:E98"/><mergeCell ref="D87:E87"/><mergeCell ref="D97:E97"/><mergeCell ref="T109:U109"/><mergeCell ref="R107:S107"/><mergeCell ref="R108:S108"/><mergeCell ref="R104:S104"/><mergeCell ref="R106:S106"/><mergeCell ref="R105:S105"/><mergeCell ref="T108:U108"/><mergeCell ref="D103:E103"/><mergeCell ref="D102:E102"/><mergeCell ref="M100:O100"/><mergeCell ref="D77:E77"/><mergeCell ref="D79:E79"/><mergeCell ref="M98:N98"/><mergeCell ref="D81:E81"/><mergeCell ref="D82:E82"/><mergeCell ref="D80:E80"/><mergeCell ref="D78:E78"/><mergeCell ref="D84:E84"/></mergeCells><pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/><pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/><drawing r:id="rId2"/></worksheet>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:W145"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" style="3" customWidth="1"/>
+    <col min="7" max="9" width="12.6640625" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="11.5546875" style="3" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.6640625" style="4" customWidth="1"/>
+    <col min="16" max="19" width="11.6640625" style="3" customWidth="1"/>
+    <col min="20" max="20" width="13.88671875" customWidth="1"/>
+    <col min="21" max="21" width="14" customWidth="1"/>
+    <col min="22" max="22" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRISTIAN</t>
+        </is>
+      </c>
+      <c r="C1" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRISTIAN</t>
+        </is>
+      </c>
+      <c r="D1" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PEDRO</t>
+        </is>
+      </c>
+      <c r="E1" s="111"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="119"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="111"/>
+      <c r="R1" s="111"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="113"/>
+    </row>
+    <row r="2" spans="1:23" s="8" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="111"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="119"/>
+      <c r="K2" s="119"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="111"/>
+      <c r="R2" s="120"/>
+      <c r="S2" s="119"/>
+      <c r="T2" s="119"/>
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+      <c r="W2" s="113"/>
+    </row>
+    <row r="3" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="121" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
+      <c r="H3" s="119"/>
+      <c r="I3" s="119"/>
+      <c r="J3" s="119"/>
+      <c r="K3" s="119"/>
+      <c r="L3" s="119"/>
+      <c r="M3" s="119"/>
+      <c r="N3" s="119"/>
+      <c r="O3" s="119"/>
+      <c r="P3" s="119"/>
+      <c r="Q3" s="119"/>
+      <c r="R3" s="119"/>
+      <c r="S3" s="119"/>
+      <c r="T3" s="119"/>
+      <c r="U3" s="109"/>
+      <c r="V3" s="162"/>
+      <c r="W3" s="115"/>
+    </row>
+    <row r="4" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="121" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="119"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="119"/>
+      <c r="J4" s="119"/>
+      <c r="K4" s="119"/>
+      <c r="L4" s="119"/>
+      <c r="M4" s="119"/>
+      <c r="N4" s="119"/>
+      <c r="O4" s="119"/>
+      <c r="P4" s="119"/>
+      <c r="Q4" s="119"/>
+      <c r="R4" s="119"/>
+      <c r="S4" s="119"/>
+      <c r="T4" s="119"/>
+      <c r="U4" s="109"/>
+      <c r="V4" s="162"/>
+      <c r="W4" s="115"/>
+    </row>
+    <row r="5" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="121" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">260006341</t>
+        </is>
+      </c>
+      <c r="C5" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">260006342</t>
+        </is>
+      </c>
+      <c r="D5" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">260006320</t>
+        </is>
+      </c>
+      <c r="E5" s="128"/>
+      <c r="F5" s="128"/>
+      <c r="G5" s="128"/>
+      <c r="H5" s="128"/>
+      <c r="I5" s="128"/>
+      <c r="J5" s="128"/>
+      <c r="K5" s="128"/>
+      <c r="L5" s="128"/>
+      <c r="M5" s="128"/>
+      <c r="N5" s="128"/>
+      <c r="O5" s="128"/>
+      <c r="P5" s="128"/>
+      <c r="Q5" s="128"/>
+      <c r="R5" s="119"/>
+      <c r="S5" s="119"/>
+      <c r="T5" s="119"/>
+      <c r="U5" s="110"/>
+      <c r="V5" s="110"/>
+      <c r="W5" s="110"/>
+    </row>
+    <row r="6" spans="1:23" s="44" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="121" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="119">
+        <v>5</v>
+      </c>
+      <c r="C6" s="119">
+        <v>5</v>
+      </c>
+      <c r="D6" s="119">
+        <v>5</v>
+      </c>
+      <c r="E6" s="119"/>
+      <c r="F6" s="119"/>
+      <c r="G6" s="119"/>
+      <c r="H6" s="119"/>
+      <c r="I6" s="119"/>
+      <c r="J6" s="119"/>
+      <c r="K6" s="119"/>
+      <c r="L6" s="119"/>
+      <c r="M6" s="110"/>
+      <c r="N6" s="110"/>
+      <c r="O6" s="110"/>
+      <c r="P6" s="110"/>
+      <c r="Q6" s="110"/>
+      <c r="R6" s="119"/>
+      <c r="S6" s="119"/>
+      <c r="T6" s="119"/>
+      <c r="U6" s="110"/>
+      <c r="V6" s="110"/>
+      <c r="W6" s="110"/>
+    </row>
+    <row r="7" spans="1:23" s="44" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="121" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="163">
+        <v>1000000</v>
+      </c>
+      <c r="C7" s="163">
+        <v>1000000</v>
+      </c>
+      <c r="D7" s="163">
+        <v>1054260</v>
+      </c>
+      <c r="E7" s="163"/>
+      <c r="F7" s="163"/>
+      <c r="G7" s="163"/>
+      <c r="H7" s="163"/>
+      <c r="I7" s="163"/>
+      <c r="J7" s="163"/>
+      <c r="K7" s="163"/>
+      <c r="L7" s="163"/>
+      <c r="M7" s="163"/>
+      <c r="N7" s="163"/>
+      <c r="O7" s="163"/>
+      <c r="P7" s="163"/>
+      <c r="Q7" s="163"/>
+      <c r="R7" s="155"/>
+      <c r="S7" s="155"/>
+      <c r="T7" s="155"/>
+      <c r="U7" s="156"/>
+      <c r="V7" s="156"/>
+      <c r="W7" s="156"/>
+    </row>
+    <row r="8" spans="1:23" s="44" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="111"/>
+      <c r="B8" s="156"/>
+      <c r="C8" s="110"/>
+      <c r="D8" s="156"/>
+      <c r="E8" s="110"/>
+      <c r="F8" s="109"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="156"/>
+      <c r="I8" s="110"/>
+      <c r="J8" s="156"/>
+      <c r="K8" s="110"/>
+      <c r="L8" s="109"/>
+      <c r="M8" s="110"/>
+      <c r="N8" s="109"/>
+      <c r="O8" s="110"/>
+      <c r="P8" s="157"/>
+      <c r="Q8" s="110"/>
+      <c r="R8" s="157"/>
+      <c r="S8" s="110"/>
+      <c r="T8" s="157"/>
+      <c r="U8" s="110"/>
+      <c r="V8" s="109"/>
+      <c r="W8" s="110"/>
+    </row>
+    <row r="9" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="112" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="164"/>
+      <c r="C9" s="164"/>
+      <c r="D9" s="164"/>
+      <c r="E9" s="156"/>
+      <c r="F9" s="109"/>
+      <c r="G9" s="156"/>
+      <c r="H9" s="109"/>
+      <c r="I9" s="156"/>
+      <c r="J9" s="109"/>
+      <c r="K9" s="156"/>
+      <c r="L9" s="109"/>
+      <c r="M9" s="156"/>
+      <c r="N9" s="109"/>
+      <c r="O9" s="156"/>
+      <c r="P9" s="157"/>
+      <c r="Q9" s="156"/>
+      <c r="R9" s="157"/>
+      <c r="S9" s="158"/>
+      <c r="T9" s="158"/>
+      <c r="U9" s="156"/>
+      <c r="V9" s="109"/>
+      <c r="W9" s="156"/>
+    </row>
+    <row r="10" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="112" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="164"/>
+      <c r="C10" s="164"/>
+      <c r="D10" s="164"/>
+      <c r="E10" s="156"/>
+      <c r="F10" s="109"/>
+      <c r="G10" s="156"/>
+      <c r="H10" s="109"/>
+      <c r="I10" s="156"/>
+      <c r="J10" s="109"/>
+      <c r="K10" s="156"/>
+      <c r="L10" s="109"/>
+      <c r="M10" s="156"/>
+      <c r="N10" s="109"/>
+      <c r="O10" s="156"/>
+      <c r="P10" s="157"/>
+      <c r="Q10" s="156"/>
+      <c r="R10" s="157"/>
+      <c r="S10" s="158"/>
+      <c r="T10" s="158"/>
+      <c r="U10" s="156"/>
+      <c r="V10" s="109"/>
+      <c r="W10" s="156"/>
+    </row>
+    <row r="11" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="112" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="164"/>
+      <c r="C11" s="164"/>
+      <c r="D11" s="164"/>
+      <c r="E11" s="156"/>
+      <c r="F11" s="109"/>
+      <c r="G11" s="156"/>
+      <c r="H11" s="109"/>
+      <c r="I11" s="156"/>
+      <c r="J11" s="109"/>
+      <c r="K11" s="156"/>
+      <c r="L11" s="109"/>
+      <c r="M11" s="156"/>
+      <c r="N11" s="109"/>
+      <c r="O11" s="156"/>
+      <c r="P11" s="157"/>
+      <c r="Q11" s="156"/>
+      <c r="R11" s="157"/>
+      <c r="S11" s="158"/>
+      <c r="T11" s="158"/>
+      <c r="U11" s="156"/>
+      <c r="V11" s="109"/>
+      <c r="W11" s="156"/>
+    </row>
+    <row r="12" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="112" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="164">
+        <v>127092</v>
+      </c>
+      <c r="C12" s="164">
+        <v>972618</v>
+      </c>
+      <c r="D12" s="164">
+        <v>461001</v>
+      </c>
+      <c r="E12" s="156"/>
+      <c r="F12" s="109"/>
+      <c r="G12" s="156"/>
+      <c r="H12" s="109"/>
+      <c r="I12" s="156"/>
+      <c r="J12" s="109"/>
+      <c r="K12" s="156"/>
+      <c r="L12" s="109"/>
+      <c r="M12" s="156"/>
+      <c r="N12" s="109"/>
+      <c r="O12" s="156"/>
+      <c r="P12" s="157"/>
+      <c r="Q12" s="156"/>
+      <c r="R12" s="157"/>
+      <c r="S12" s="158"/>
+      <c r="T12" s="158"/>
+      <c r="U12" s="156"/>
+      <c r="V12" s="109"/>
+      <c r="W12" s="156"/>
+    </row>
+    <row r="13" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="112" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="164"/>
+      <c r="C13" s="164"/>
+      <c r="D13" s="164"/>
+      <c r="E13" s="156"/>
+      <c r="F13" s="109"/>
+      <c r="G13" s="156"/>
+      <c r="H13" s="109"/>
+      <c r="I13" s="156"/>
+      <c r="J13" s="109"/>
+      <c r="K13" s="156"/>
+      <c r="L13" s="109"/>
+      <c r="M13" s="156"/>
+      <c r="N13" s="109"/>
+      <c r="O13" s="156"/>
+      <c r="P13" s="157"/>
+      <c r="Q13" s="156"/>
+      <c r="R13" s="157"/>
+      <c r="S13" s="158"/>
+      <c r="T13" s="158"/>
+      <c r="U13" s="156"/>
+      <c r="V13" s="109"/>
+      <c r="W13" s="156"/>
+    </row>
+    <row r="14" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="112" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="164"/>
+      <c r="C14" s="164"/>
+      <c r="D14" s="164"/>
+      <c r="E14" s="156"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="156"/>
+      <c r="H14" s="109"/>
+      <c r="I14" s="156"/>
+      <c r="J14" s="109"/>
+      <c r="K14" s="156"/>
+      <c r="L14" s="109"/>
+      <c r="M14" s="156"/>
+      <c r="N14" s="109"/>
+      <c r="O14" s="156"/>
+      <c r="P14" s="157"/>
+      <c r="Q14" s="156"/>
+      <c r="R14" s="157"/>
+      <c r="S14" s="158"/>
+      <c r="T14" s="158"/>
+      <c r="U14" s="156"/>
+      <c r="V14" s="109"/>
+      <c r="W14" s="156"/>
+    </row>
+    <row r="15" spans="1:23" s="160" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="112" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="164"/>
+      <c r="C15" s="164"/>
+      <c r="D15" s="164"/>
+      <c r="E15" s="156"/>
+      <c r="F15" s="109"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="109"/>
+      <c r="I15" s="156"/>
+      <c r="J15" s="109"/>
+      <c r="K15" s="156"/>
+      <c r="L15" s="109"/>
+      <c r="M15" s="156"/>
+      <c r="N15" s="109"/>
+      <c r="O15" s="156"/>
+      <c r="P15" s="157"/>
+      <c r="Q15" s="156"/>
+      <c r="R15" s="157"/>
+      <c r="S15" s="158"/>
+      <c r="T15" s="158"/>
+      <c r="U15" s="156"/>
+      <c r="V15" s="109"/>
+      <c r="W15" s="156"/>
+    </row>
+    <row r="16" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="112" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="164"/>
+      <c r="C16" s="164"/>
+      <c r="D16" s="164"/>
+      <c r="E16" s="156"/>
+      <c r="F16" s="109"/>
+      <c r="G16" s="156"/>
+      <c r="H16" s="109"/>
+      <c r="I16" s="159"/>
+      <c r="J16" s="109"/>
+      <c r="K16" s="159"/>
+      <c r="L16" s="109"/>
+      <c r="M16" s="156"/>
+      <c r="N16" s="109"/>
+      <c r="O16" s="156"/>
+      <c r="P16" s="157"/>
+      <c r="Q16" s="156"/>
+      <c r="R16" s="157"/>
+      <c r="S16" s="158"/>
+      <c r="T16" s="158"/>
+      <c r="U16" s="156"/>
+      <c r="V16" s="109"/>
+      <c r="W16" s="156"/>
+    </row>
+    <row r="17" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="112" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="164"/>
+      <c r="C17" s="164"/>
+      <c r="D17" s="164"/>
+      <c r="E17" s="156"/>
+      <c r="F17" s="109"/>
+      <c r="G17" s="156"/>
+      <c r="H17" s="109"/>
+      <c r="I17" s="159"/>
+      <c r="J17" s="109"/>
+      <c r="K17" s="156"/>
+      <c r="L17" s="109"/>
+      <c r="M17" s="156"/>
+      <c r="N17" s="109"/>
+      <c r="O17" s="156"/>
+      <c r="P17" s="157"/>
+      <c r="Q17" s="156"/>
+      <c r="R17" s="157"/>
+      <c r="S17" s="158"/>
+      <c r="T17" s="158"/>
+      <c r="U17" s="156"/>
+      <c r="V17" s="109"/>
+      <c r="W17" s="156"/>
+    </row>
+    <row r="18" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="112" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="109">
+        <f>SUM(B9:B17)</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="109">
+        <f t="shared" ref="C18:O18" si="0">SUM(C9:C17)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O18" s="109">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P18" s="109">
+        <f t="shared" ref="P18" si="1">SUM(P9:P17)</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="109">
+        <f>SUM(Q9:Q17)</f>
+        <v>0</v>
+      </c>
+      <c r="R18" s="109">
+        <f>SUM(R9:R17)</f>
+        <v>0</v>
+      </c>
+      <c r="S18" s="115">
+        <f>SUM(S9:S17)</f>
+        <v>0</v>
+      </c>
+      <c r="T18" s="115">
+        <f>SUM(T9:T17)</f>
+        <v>0</v>
+      </c>
+      <c r="U18" s="109">
+        <f t="shared" ref="U18:W18" si="2">SUM(U9:U17)</f>
+        <v>0</v>
+      </c>
+      <c r="V18" s="109">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W18" s="109">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="112"/>
+      <c r="B19" s="109"/>
+      <c r="C19" s="109"/>
+      <c r="D19" s="109"/>
+      <c r="E19" s="109"/>
+      <c r="F19" s="156"/>
+      <c r="G19" s="109"/>
+      <c r="H19" s="109"/>
+      <c r="I19" s="109"/>
+      <c r="J19" s="109"/>
+      <c r="K19" s="109"/>
+      <c r="L19" s="109"/>
+      <c r="M19" s="109"/>
+      <c r="N19" s="109"/>
+      <c r="O19" s="109"/>
+      <c r="P19" s="109"/>
+      <c r="Q19" s="109"/>
+      <c r="R19" s="109"/>
+      <c r="S19" s="115"/>
+      <c r="T19" s="115"/>
+      <c r="U19" s="109"/>
+      <c r="V19" s="109"/>
+      <c r="W19" s="109"/>
+    </row>
+    <row r="20" spans="1:23" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="112" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="109" t="e">
+        <f t="shared" ref="B20:O20" si="3">B18-B7</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="L20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O20" s="109">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P20" s="109">
+        <f t="shared" ref="P20" si="4">P18-P7</f>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="109">
+        <f>Q18-Q7</f>
+        <v>0</v>
+      </c>
+      <c r="R20" s="109">
+        <f>R18-R7</f>
+        <v>0</v>
+      </c>
+      <c r="S20" s="109">
+        <f>S18-S7</f>
+        <v>0</v>
+      </c>
+      <c r="T20" s="109">
+        <f>T18-T7</f>
+        <v>0</v>
+      </c>
+      <c r="U20" s="109">
+        <f t="shared" ref="U20:W20" si="5">U18-U7</f>
+        <v>0</v>
+      </c>
+      <c r="V20" s="109">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W20" s="109">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="9"/>
+    </row>
+    <row r="22" spans="1:23" s="1" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D22" s="2"/>
+      <c r="M22" s="177" t="s">
+        <v>48</v>
+      </c>
+      <c r="N22" s="177"/>
+      <c r="O22" s="177"/>
+      <c r="P22" s="177"/>
+      <c r="Q22" s="177"/>
+      <c r="R22" s="177"/>
+      <c r="S22" s="177"/>
+      <c r="T22" s="177"/>
+      <c r="U22" s="177"/>
+    </row>
+    <row r="23" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D23" s="6"/>
+      <c r="J23"/>
+      <c r="L23"/>
+      <c r="M23" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="N23" s="184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30-06-2026</t>
+        </is>
+      </c>
+      <c r="O23" s="185"/>
+      <c r="P23" s="185"/>
+      <c r="Q23" s="185"/>
+      <c r="R23" s="185"/>
+      <c r="S23" s="186"/>
+      <c r="T23" s="118" t="s">
+        <v>38</v>
+      </c>
+      <c r="U23" s="105">
+        <v>15</v>
+      </c>
+      <c r="W23" s="90" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="2"/>
+      <c r="C24" s="18"/>
+      <c r="J24"/>
+      <c r="K24" s="15"/>
+      <c r="L24"/>
+      <c r="M24" s="16"/>
+      <c r="N24" s="187" t="s">
+        <v>49</v>
+      </c>
+      <c r="O24" s="188"/>
+      <c r="P24" s="188"/>
+      <c r="Q24" s="188"/>
+      <c r="R24" s="188"/>
+      <c r="S24" s="189"/>
+      <c r="T24" s="107" t="s">
+        <v>11</v>
+      </c>
+      <c r="U24" s="106">
+        <v>3054260</v>
+      </c>
+      <c r="W24" s="117">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B25" s="2"/>
+      <c r="C25" s="102"/>
+      <c r="D25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="J25"/>
+      <c r="L25"/>
+      <c r="M25" s="165" t="s">
+        <v>16</v>
+      </c>
+      <c r="N25" s="166"/>
+      <c r="O25" s="147"/>
+      <c r="P25" s="148"/>
+      <c r="Q25" s="144"/>
+      <c r="R25" s="145"/>
+      <c r="S25" s="146"/>
+      <c r="T25" s="190" t="s">
+        <v>17</v>
+      </c>
+      <c r="U25" s="191"/>
+      <c r="V25" s="13"/>
+      <c r="W25" s="81" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="E26" s="4"/>
+      <c r="J26"/>
+      <c r="L26"/>
+      <c r="M26" s="78" t="s">
+        <v>53</v>
+      </c>
+      <c r="N26" s="79"/>
+      <c r="O26" s="125"/>
+      <c r="P26" s="126"/>
+      <c r="Q26" s="169"/>
+      <c r="R26" s="170"/>
+      <c r="S26" s="171"/>
+      <c r="T26" s="123"/>
+      <c r="U26" s="124"/>
+      <c r="V26" s="13"/>
+      <c r="W26" s="81"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="I27" s="108" t="str">
+        <f>B$1</f>
+      </c>
+      <c r="J27" s="135" t="str">
+        <f>B9</f>
+      </c>
+      <c r="L27"/>
+      <c r="M27" s="78" t="s">
+        <v>18</v>
+      </c>
+      <c r="N27" s="79"/>
+      <c r="O27" s="167"/>
+      <c r="P27" s="176"/>
+      <c r="Q27" s="169"/>
+      <c r="R27" s="170"/>
+      <c r="S27" s="171"/>
+      <c r="T27" s="182" t="s">
+        <v>19</v>
+      </c>
+      <c r="U27" s="183"/>
+      <c r="V27" s="19"/>
+      <c r="W27" s="91">
+        <v>3054260</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="I28" s="108">
+        <f>C$1</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="135">
+        <f>C9</f>
+        <v>0</v>
+      </c>
+      <c r="L28"/>
+      <c r="M28" s="174" t="s">
+        <v>20</v>
+      </c>
+      <c r="N28" s="175"/>
+      <c r="O28" s="167"/>
+      <c r="P28" s="176"/>
+      <c r="Q28" s="169">
+        <v>1560711</v>
+      </c>
+      <c r="R28" s="170"/>
+      <c r="S28" s="171"/>
+      <c r="T28" s="180" t="s">
+        <v>39</v>
+      </c>
+      <c r="U28" s="181"/>
+      <c r="V28" s="21"/>
+      <c r="W28" s="13"/>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="I29" s="108">
+        <f>D$1</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="135">
+        <f>D9</f>
+        <v>0</v>
+      </c>
+      <c r="K29" s="24"/>
+      <c r="L29"/>
+      <c r="M29" s="174" t="s">
+        <v>21</v>
+      </c>
+      <c r="N29" s="175"/>
+      <c r="O29" s="167"/>
+      <c r="P29" s="176"/>
+      <c r="Q29" s="169"/>
+      <c r="R29" s="170"/>
+      <c r="S29" s="171"/>
+      <c r="T29" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="U29" s="179"/>
+      <c r="W29" s="92" t="str">
+        <f>U23</f>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A30" s="1"/>
+      <c r="I30" s="108">
+        <f>E$1</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="135">
+        <f>E9</f>
+        <v>0</v>
+      </c>
+      <c r="L30"/>
+      <c r="M30" s="174" t="s">
+        <v>22</v>
+      </c>
+      <c r="N30" s="175"/>
+      <c r="O30" s="167"/>
+      <c r="P30" s="168"/>
+      <c r="Q30" s="169"/>
+      <c r="R30" s="170"/>
+      <c r="S30" s="171"/>
+      <c r="T30" s="172" t="s">
+        <v>41</v>
+      </c>
+      <c r="U30" s="173"/>
+      <c r="V30" s="24"/>
+      <c r="W30" s="21" t="str">
+        <f>Q34</f>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A31" s="1"/>
+      <c r="I31" s="108">
+        <f>F$1</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="135">
+        <f>F9</f>
+        <v>0</v>
+      </c>
+      <c r="L31"/>
+      <c r="M31" s="174" t="s">
+        <v>23</v>
+      </c>
+      <c r="N31" s="175"/>
+      <c r="O31" s="167"/>
+      <c r="P31" s="176"/>
+      <c r="Q31" s="169"/>
+      <c r="R31" s="170"/>
+      <c r="S31" s="171"/>
+      <c r="T31" s="28"/>
+      <c r="U31" s="26"/>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A32" s="1"/>
+      <c r="I32" s="108">
+        <f>G$1</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="135">
+        <f>G9</f>
+        <v>0</v>
+      </c>
+      <c r="L32"/>
+      <c r="M32" s="174" t="s">
+        <v>24</v>
+      </c>
+      <c r="N32" s="175"/>
+      <c r="O32" s="167"/>
+      <c r="P32" s="176"/>
+      <c r="Q32" s="169"/>
+      <c r="R32" s="170"/>
+      <c r="S32" s="171"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="26"/>
+      <c r="W32" s="81" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A33" s="1"/>
+      <c r="I33" s="108">
+        <f>H$1</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="135">
+        <f>H9</f>
+        <v>0</v>
+      </c>
+      <c r="L33"/>
+      <c r="M33" s="78" t="s">
+        <v>25</v>
+      </c>
+      <c r="N33" s="80"/>
+      <c r="O33" s="167"/>
+      <c r="P33" s="176"/>
+      <c r="Q33" s="169"/>
+      <c r="R33" s="170"/>
+      <c r="S33" s="171"/>
+      <c r="T33" s="28"/>
+      <c r="U33" s="26"/>
+      <c r="W33" s="116" t="e">
+        <f>W30-W27</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="1"/>
+      <c r="I34" s="108">
+        <f>I$1</f>
+        <v>0</v>
+      </c>
+      <c r="J34" s="135">
+        <f>I9</f>
+        <v>0</v>
+      </c>
+      <c r="L34" s="8"/>
+      <c r="M34" s="195" t="s">
+        <v>26</v>
+      </c>
+      <c r="N34" s="196"/>
+      <c r="O34" s="197"/>
+      <c r="P34" s="198"/>
+      <c r="Q34" s="169"/>
+      <c r="R34" s="170"/>
+      <c r="S34" s="171"/>
+      <c r="T34" s="30"/>
+      <c r="U34" s="29"/>
+      <c r="V34" s="1"/>
+      <c r="W34" s="24"/>
+    </row>
+    <row r="35" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="1"/>
+      <c r="D35" s="31"/>
+      <c r="I35" s="108">
+        <f>J$1</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="27">
+        <f>J9</f>
+        <v>0</v>
+      </c>
+      <c r="L35"/>
+      <c r="M35" s="199" t="s">
+        <v>27</v>
+      </c>
+      <c r="N35" s="200"/>
+      <c r="O35" s="201"/>
+      <c r="P35" s="193" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q35" s="194"/>
+      <c r="R35" s="193" t="s">
+        <v>29</v>
+      </c>
+      <c r="S35" s="194"/>
+      <c r="T35" s="193" t="s">
+        <v>30</v>
+      </c>
+      <c r="U35" s="194"/>
+      <c r="V35" s="1"/>
+      <c r="W35" s="1"/>
+    </row>
+    <row r="36" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="9"/>
+      <c r="I36" s="108">
+        <f>K$1</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="27">
+        <f>K9</f>
+        <v>0</v>
+      </c>
+      <c r="L36"/>
+      <c r="M36" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="N36" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="O36" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="P36" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q36" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="R36" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="S36" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="T36" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="U36" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="V36" s="1"/>
+      <c r="W36" s="1"/>
+    </row>
+    <row r="37" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="M37" s="37"/>
+      <c r="N37" s="38"/>
+      <c r="O37" s="39"/>
+      <c r="P37" s="150">
+        <v>605655</v>
+      </c>
+      <c r="Q37" s="76">
+        <v>10000</v>
+      </c>
+      <c r="R37" s="152"/>
+      <c r="S37" s="77"/>
+      <c r="T37" s="151"/>
+      <c r="U37" s="73"/>
+      <c r="A37" s="1"/>
+      <c r="I37" s="108">
+        <f>L$1</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="27">
+        <f>L9</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="24"/>
+      <c r="L37"/>
+      <c r="V37" s="1"/>
+      <c r="W37" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M38" s="37"/>
+      <c r="N38" s="38"/>
+      <c r="O38" s="39"/>
+      <c r="P38" s="151">
+        <v>605656</v>
+      </c>
+      <c r="Q38" s="65">
+        <v>10001</v>
+      </c>
+      <c r="R38" s="153"/>
+      <c r="S38" s="73"/>
+      <c r="T38" s="151"/>
+      <c r="U38" s="67"/>
+      <c r="A38" s="1"/>
+      <c r="I38" s="108"/>
+      <c r="J38" s="27"/>
+      <c r="K38" s="24"/>
+      <c r="L38" s="104"/>
+      <c r="V38" s="1"/>
+      <c r="W38" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M39" s="37"/>
+      <c r="N39" s="38"/>
+      <c r="O39" s="39"/>
+      <c r="P39" s="151">
+        <v>605657</v>
+      </c>
+      <c r="Q39" s="65">
+        <v>10002</v>
+      </c>
+      <c r="R39" s="153"/>
+      <c r="S39" s="73"/>
+      <c r="T39" s="151"/>
+      <c r="U39" s="67"/>
+      <c r="A39" s="1"/>
+      <c r="I39" s="108"/>
+      <c r="J39" s="27"/>
+      <c r="K39" s="24"/>
+      <c r="L39" s="104"/>
+      <c r="V39" s="1"/>
+      <c r="W39" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M40" s="37"/>
+      <c r="N40" s="38"/>
+      <c r="O40" s="39"/>
+      <c r="P40" s="151">
+        <v>605658</v>
+      </c>
+      <c r="Q40" s="65">
+        <v>10003</v>
+      </c>
+      <c r="R40" s="153"/>
+      <c r="S40" s="73"/>
+      <c r="T40" s="151"/>
+      <c r="U40" s="67"/>
+      <c r="A40" s="1"/>
+      <c r="I40" s="108"/>
+      <c r="J40" s="27"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="104"/>
+      <c r="V40" s="1"/>
+      <c r="W40" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M41" s="37"/>
+      <c r="N41" s="38"/>
+      <c r="O41" s="39"/>
+      <c r="P41" s="151">
+        <v>605659</v>
+      </c>
+      <c r="Q41" s="65">
+        <v>10004</v>
+      </c>
+      <c r="R41" s="153"/>
+      <c r="S41" s="73"/>
+      <c r="T41" s="151"/>
+      <c r="U41" s="67"/>
+      <c r="A41" s="1"/>
+      <c r="I41" s="108"/>
+      <c r="J41" s="27"/>
+      <c r="K41" s="24"/>
+      <c r="L41" s="104"/>
+      <c r="V41" s="1"/>
+      <c r="W41" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M42" s="37"/>
+      <c r="N42" s="38"/>
+      <c r="O42" s="39"/>
+      <c r="P42" s="151">
+        <v>605660</v>
+      </c>
+      <c r="Q42" s="65">
+        <v>10005</v>
+      </c>
+      <c r="R42" s="153"/>
+      <c r="S42" s="73"/>
+      <c r="T42" s="151"/>
+      <c r="U42" s="67"/>
+      <c r="A42" s="1"/>
+      <c r="I42" s="108"/>
+      <c r="J42" s="27"/>
+      <c r="K42" s="24"/>
+      <c r="L42" s="104"/>
+      <c r="V42" s="1"/>
+      <c r="W42" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M43" s="37"/>
+      <c r="N43" s="38"/>
+      <c r="O43" s="39"/>
+      <c r="P43" s="151">
+        <v>605661</v>
+      </c>
+      <c r="Q43" s="65">
+        <v>10006</v>
+      </c>
+      <c r="R43" s="153"/>
+      <c r="S43" s="73"/>
+      <c r="T43" s="151"/>
+      <c r="U43" s="67"/>
+      <c r="A43" s="1"/>
+      <c r="I43" s="108"/>
+      <c r="J43" s="27"/>
+      <c r="K43" s="24"/>
+      <c r="L43" s="104"/>
+      <c r="V43" s="1"/>
+      <c r="W43" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M44" s="37"/>
+      <c r="N44" s="38"/>
+      <c r="O44" s="39"/>
+      <c r="P44" s="151">
+        <v>605662</v>
+      </c>
+      <c r="Q44" s="65">
+        <v>10007</v>
+      </c>
+      <c r="R44" s="153"/>
+      <c r="S44" s="73"/>
+      <c r="T44" s="151"/>
+      <c r="U44" s="67"/>
+      <c r="A44" s="1"/>
+      <c r="I44" s="108"/>
+      <c r="J44" s="27"/>
+      <c r="K44" s="24"/>
+      <c r="L44" s="104"/>
+      <c r="V44" s="1"/>
+      <c r="W44" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M45" s="37"/>
+      <c r="N45" s="38"/>
+      <c r="O45" s="39"/>
+      <c r="P45" s="151">
+        <v>605663</v>
+      </c>
+      <c r="Q45" s="65">
+        <v>10008</v>
+      </c>
+      <c r="R45" s="153"/>
+      <c r="S45" s="73"/>
+      <c r="T45" s="151"/>
+      <c r="U45" s="67"/>
+      <c r="A45" s="1"/>
+      <c r="I45" s="108"/>
+      <c r="J45" s="27"/>
+      <c r="K45" s="24"/>
+      <c r="L45" s="104"/>
+      <c r="V45" s="1"/>
+      <c r="W45" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M46" s="37"/>
+      <c r="N46" s="38"/>
+      <c r="O46" s="39"/>
+      <c r="P46" s="151">
+        <v>605664</v>
+      </c>
+      <c r="Q46" s="65">
+        <v>10009</v>
+      </c>
+      <c r="R46" s="153"/>
+      <c r="S46" s="73"/>
+      <c r="T46" s="151"/>
+      <c r="U46" s="67"/>
+      <c r="A46" s="1"/>
+      <c r="I46" s="108"/>
+      <c r="J46" s="27"/>
+      <c r="K46" s="24"/>
+      <c r="L46" s="104"/>
+      <c r="V46" s="1"/>
+      <c r="W46" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M47" s="37"/>
+      <c r="N47" s="38"/>
+      <c r="O47" s="39"/>
+      <c r="P47" s="151">
+        <v>605665</v>
+      </c>
+      <c r="Q47" s="65">
+        <v>10010</v>
+      </c>
+      <c r="R47" s="153"/>
+      <c r="S47" s="73"/>
+      <c r="T47" s="151"/>
+      <c r="U47" s="67"/>
+      <c r="A47" s="1"/>
+      <c r="I47" s="108"/>
+      <c r="J47" s="27"/>
+      <c r="K47" s="24"/>
+      <c r="L47" s="104"/>
+      <c r="V47" s="1"/>
+      <c r="W47" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M48" s="37"/>
+      <c r="N48" s="38"/>
+      <c r="O48" s="39"/>
+      <c r="P48" s="151">
+        <v>605666</v>
+      </c>
+      <c r="Q48" s="65">
+        <v>10011</v>
+      </c>
+      <c r="R48" s="153"/>
+      <c r="S48" s="73"/>
+      <c r="T48" s="151"/>
+      <c r="U48" s="67"/>
+      <c r="A48" s="1"/>
+      <c r="I48" s="108"/>
+      <c r="J48" s="27"/>
+      <c r="K48" s="24"/>
+      <c r="L48" s="104"/>
+      <c r="V48" s="1"/>
+      <c r="W48" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M49" s="37"/>
+      <c r="N49" s="38"/>
+      <c r="O49" s="39"/>
+      <c r="P49" s="151">
+        <v>605667</v>
+      </c>
+      <c r="Q49" s="65">
+        <v>10012</v>
+      </c>
+      <c r="R49" s="153"/>
+      <c r="S49" s="73"/>
+      <c r="T49" s="151"/>
+      <c r="U49" s="67"/>
+      <c r="A49" s="1"/>
+      <c r="I49" s="108"/>
+      <c r="J49" s="27"/>
+      <c r="K49" s="24"/>
+      <c r="L49" s="104"/>
+      <c r="V49" s="1"/>
+      <c r="W49" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M50" s="37"/>
+      <c r="N50" s="38"/>
+      <c r="O50" s="39"/>
+      <c r="P50" s="151">
+        <v>605668</v>
+      </c>
+      <c r="Q50" s="65">
+        <v>10013</v>
+      </c>
+      <c r="R50" s="153"/>
+      <c r="S50" s="73"/>
+      <c r="T50" s="151"/>
+      <c r="U50" s="67"/>
+      <c r="A50" s="1"/>
+      <c r="I50" s="108"/>
+      <c r="J50" s="27"/>
+      <c r="K50" s="24"/>
+      <c r="L50" s="104"/>
+      <c r="V50" s="1"/>
+      <c r="W50" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M51" s="37"/>
+      <c r="N51" s="38"/>
+      <c r="O51" s="39"/>
+      <c r="P51" s="151">
+        <v>605669</v>
+      </c>
+      <c r="Q51" s="65">
+        <v>10014</v>
+      </c>
+      <c r="R51" s="153"/>
+      <c r="S51" s="73"/>
+      <c r="T51" s="151"/>
+      <c r="U51" s="67"/>
+      <c r="A51" s="1"/>
+      <c r="I51" s="108"/>
+      <c r="J51" s="27"/>
+      <c r="K51" s="24"/>
+      <c r="L51" s="104"/>
+      <c r="V51" s="1"/>
+      <c r="W51" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M52" s="37"/>
+      <c r="N52" s="38"/>
+      <c r="O52" s="39"/>
+      <c r="P52" s="151">
+        <v>605670</v>
+      </c>
+      <c r="Q52" s="65">
+        <v>10015</v>
+      </c>
+      <c r="R52" s="153"/>
+      <c r="S52" s="73"/>
+      <c r="T52" s="151"/>
+      <c r="U52" s="67"/>
+      <c r="A52" s="1"/>
+      <c r="I52" s="108"/>
+      <c r="J52" s="27"/>
+      <c r="K52" s="24"/>
+      <c r="L52" s="104"/>
+      <c r="V52" s="1"/>
+      <c r="W52" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M53" s="37"/>
+      <c r="N53" s="38"/>
+      <c r="O53" s="39"/>
+      <c r="P53" s="151">
+        <v>605671</v>
+      </c>
+      <c r="Q53" s="65">
+        <v>10016</v>
+      </c>
+      <c r="R53" s="153"/>
+      <c r="S53" s="73"/>
+      <c r="T53" s="151"/>
+      <c r="U53" s="67"/>
+      <c r="A53" s="1"/>
+      <c r="I53" s="108"/>
+      <c r="J53" s="27"/>
+      <c r="K53" s="24"/>
+      <c r="L53" s="104"/>
+      <c r="V53" s="1"/>
+      <c r="W53" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M54" s="37"/>
+      <c r="N54" s="38"/>
+      <c r="O54" s="39"/>
+      <c r="P54" s="151">
+        <v>605655</v>
+      </c>
+      <c r="Q54" s="65">
+        <v>10000</v>
+      </c>
+      <c r="R54" s="153"/>
+      <c r="S54" s="73"/>
+      <c r="T54" s="151"/>
+      <c r="U54" s="67"/>
+      <c r="A54" s="1"/>
+      <c r="I54" s="108"/>
+      <c r="J54" s="27"/>
+      <c r="K54" s="24"/>
+      <c r="L54" s="104"/>
+      <c r="V54" s="1"/>
+      <c r="W54" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M55" s="37"/>
+      <c r="N55" s="38"/>
+      <c r="O55" s="39"/>
+      <c r="P55" s="151">
+        <v>605656</v>
+      </c>
+      <c r="Q55" s="65">
+        <v>10001</v>
+      </c>
+      <c r="R55" s="153"/>
+      <c r="S55" s="73"/>
+      <c r="T55" s="151"/>
+      <c r="U55" s="67"/>
+      <c r="A55" s="1"/>
+      <c r="I55" s="108"/>
+      <c r="J55" s="27"/>
+      <c r="K55" s="24"/>
+      <c r="L55" s="104"/>
+      <c r="V55" s="1"/>
+      <c r="W55" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M56" s="37"/>
+      <c r="N56" s="38"/>
+      <c r="O56" s="39"/>
+      <c r="P56" s="151">
+        <v>605657</v>
+      </c>
+      <c r="Q56" s="65">
+        <v>10002</v>
+      </c>
+      <c r="R56" s="153"/>
+      <c r="S56" s="73"/>
+      <c r="T56" s="151"/>
+      <c r="U56" s="67"/>
+      <c r="A56" s="1"/>
+      <c r="I56" s="108"/>
+      <c r="J56" s="27"/>
+      <c r="K56" s="24"/>
+      <c r="L56" s="104"/>
+      <c r="V56" s="1"/>
+      <c r="W56" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M57" s="37"/>
+      <c r="N57" s="38"/>
+      <c r="O57" s="39"/>
+      <c r="P57" s="151">
+        <v>605658</v>
+      </c>
+      <c r="Q57" s="65">
+        <v>10003</v>
+      </c>
+      <c r="R57" s="153"/>
+      <c r="S57" s="73"/>
+      <c r="T57" s="151"/>
+      <c r="U57" s="67"/>
+      <c r="A57" s="1"/>
+      <c r="I57" s="108"/>
+      <c r="J57" s="27"/>
+      <c r="K57" s="24"/>
+      <c r="L57" s="104"/>
+      <c r="V57" s="1"/>
+      <c r="W57" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M58" s="37"/>
+      <c r="N58" s="38"/>
+      <c r="O58" s="39"/>
+      <c r="P58" s="151">
+        <v>605659</v>
+      </c>
+      <c r="Q58" s="65">
+        <v>10004</v>
+      </c>
+      <c r="R58" s="153"/>
+      <c r="S58" s="73"/>
+      <c r="T58" s="151"/>
+      <c r="U58" s="67"/>
+      <c r="A58" s="1"/>
+      <c r="I58" s="108"/>
+      <c r="J58" s="27"/>
+      <c r="K58" s="24"/>
+      <c r="L58" s="104"/>
+      <c r="V58" s="1"/>
+      <c r="W58" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M59" s="37"/>
+      <c r="N59" s="38"/>
+      <c r="O59" s="39"/>
+      <c r="P59" s="151">
+        <v>605660</v>
+      </c>
+      <c r="Q59" s="65">
+        <v>10005</v>
+      </c>
+      <c r="R59" s="153"/>
+      <c r="S59" s="73"/>
+      <c r="T59" s="151"/>
+      <c r="U59" s="67"/>
+      <c r="A59" s="1"/>
+      <c r="I59" s="108"/>
+      <c r="J59" s="27"/>
+      <c r="K59" s="24"/>
+      <c r="L59" s="104"/>
+      <c r="V59" s="1"/>
+      <c r="W59" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M60" s="37"/>
+      <c r="N60" s="38"/>
+      <c r="O60" s="39"/>
+      <c r="P60" s="151">
+        <v>605661</v>
+      </c>
+      <c r="Q60" s="65">
+        <v>10006</v>
+      </c>
+      <c r="R60" s="153"/>
+      <c r="S60" s="73"/>
+      <c r="T60" s="151"/>
+      <c r="U60" s="67"/>
+      <c r="A60" s="1"/>
+      <c r="I60" s="108"/>
+      <c r="J60" s="27"/>
+      <c r="K60" s="24"/>
+      <c r="L60" s="104"/>
+      <c r="V60" s="1"/>
+      <c r="W60" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M61" s="37"/>
+      <c r="N61" s="38"/>
+      <c r="O61" s="39"/>
+      <c r="P61" s="151">
+        <v>605662</v>
+      </c>
+      <c r="Q61" s="65">
+        <v>10007</v>
+      </c>
+      <c r="R61" s="153"/>
+      <c r="S61" s="73"/>
+      <c r="T61" s="151"/>
+      <c r="U61" s="67"/>
+      <c r="A61" s="1"/>
+      <c r="I61" s="108"/>
+      <c r="J61" s="27"/>
+      <c r="K61" s="24"/>
+      <c r="L61" s="104"/>
+      <c r="V61" s="1"/>
+      <c r="W61" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M62" s="37"/>
+      <c r="N62" s="38"/>
+      <c r="O62" s="39"/>
+      <c r="P62" s="151">
+        <v>605663</v>
+      </c>
+      <c r="Q62" s="65">
+        <v>10008</v>
+      </c>
+      <c r="R62" s="153"/>
+      <c r="S62" s="73"/>
+      <c r="T62" s="151"/>
+      <c r="U62" s="67"/>
+      <c r="A62" s="1"/>
+      <c r="I62" s="108"/>
+      <c r="J62" s="27"/>
+      <c r="K62" s="24"/>
+      <c r="L62" s="104"/>
+      <c r="V62" s="1"/>
+      <c r="W62" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M63" s="37"/>
+      <c r="N63" s="38"/>
+      <c r="O63" s="39"/>
+      <c r="P63" s="151">
+        <v>605664</v>
+      </c>
+      <c r="Q63" s="65">
+        <v>10009</v>
+      </c>
+      <c r="R63" s="153"/>
+      <c r="S63" s="73"/>
+      <c r="T63" s="151"/>
+      <c r="U63" s="67"/>
+      <c r="A63" s="1"/>
+      <c r="I63" s="108"/>
+      <c r="J63" s="27"/>
+      <c r="K63" s="24"/>
+      <c r="L63" s="104"/>
+      <c r="V63" s="1"/>
+      <c r="W63" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M64" s="37"/>
+      <c r="N64" s="38"/>
+      <c r="O64" s="39"/>
+      <c r="P64" s="151">
+        <v>605665</v>
+      </c>
+      <c r="Q64" s="65">
+        <v>10010</v>
+      </c>
+      <c r="R64" s="153"/>
+      <c r="S64" s="73"/>
+      <c r="T64" s="151"/>
+      <c r="U64" s="67"/>
+      <c r="A64" s="1"/>
+      <c r="I64" s="108"/>
+      <c r="J64" s="27"/>
+      <c r="K64" s="24"/>
+      <c r="L64" s="104"/>
+      <c r="V64" s="1"/>
+      <c r="W64" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M65" s="37"/>
+      <c r="N65" s="38"/>
+      <c r="O65" s="39"/>
+      <c r="P65" s="151">
+        <v>605666</v>
+      </c>
+      <c r="Q65" s="65">
+        <v>10011</v>
+      </c>
+      <c r="R65" s="153"/>
+      <c r="S65" s="73"/>
+      <c r="T65" s="151"/>
+      <c r="U65" s="67"/>
+      <c r="A65" s="1"/>
+      <c r="I65" s="108"/>
+      <c r="J65" s="27"/>
+      <c r="K65" s="24"/>
+      <c r="L65" s="104"/>
+      <c r="V65" s="1"/>
+      <c r="W65" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M66" s="37"/>
+      <c r="N66" s="38"/>
+      <c r="O66" s="39"/>
+      <c r="P66" s="151">
+        <v>605667</v>
+      </c>
+      <c r="Q66" s="65">
+        <v>10012</v>
+      </c>
+      <c r="R66" s="153"/>
+      <c r="S66" s="73"/>
+      <c r="T66" s="151"/>
+      <c r="U66" s="67"/>
+      <c r="A66" s="1"/>
+      <c r="I66" s="108"/>
+      <c r="J66" s="27"/>
+      <c r="K66" s="24"/>
+      <c r="L66" s="104"/>
+      <c r="V66" s="1"/>
+      <c r="W66" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M67" s="37"/>
+      <c r="N67" s="38"/>
+      <c r="O67" s="39"/>
+      <c r="P67" s="151">
+        <v>605668</v>
+      </c>
+      <c r="Q67" s="65">
+        <v>10013</v>
+      </c>
+      <c r="R67" s="153"/>
+      <c r="S67" s="73"/>
+      <c r="T67" s="151"/>
+      <c r="U67" s="67"/>
+      <c r="A67" s="1"/>
+      <c r="I67" s="108"/>
+      <c r="J67" s="27"/>
+      <c r="K67" s="24"/>
+      <c r="L67" s="104"/>
+      <c r="V67" s="1"/>
+      <c r="W67" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M68" s="37"/>
+      <c r="N68" s="38"/>
+      <c r="O68" s="39"/>
+      <c r="P68" s="151">
+        <v>605669</v>
+      </c>
+      <c r="Q68" s="65">
+        <v>10014</v>
+      </c>
+      <c r="R68" s="153"/>
+      <c r="S68" s="73"/>
+      <c r="T68" s="151"/>
+      <c r="U68" s="67"/>
+      <c r="A68" s="1"/>
+      <c r="I68" s="108"/>
+      <c r="J68" s="27"/>
+      <c r="K68" s="24"/>
+      <c r="L68" s="104"/>
+      <c r="V68" s="1"/>
+      <c r="W68" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M69" s="37"/>
+      <c r="N69" s="38"/>
+      <c r="O69" s="39"/>
+      <c r="P69" s="151">
+        <v>605670</v>
+      </c>
+      <c r="Q69" s="65">
+        <v>10015</v>
+      </c>
+      <c r="R69" s="153"/>
+      <c r="S69" s="73"/>
+      <c r="T69" s="151"/>
+      <c r="U69" s="67"/>
+      <c r="A69" s="1"/>
+      <c r="I69" s="108"/>
+      <c r="J69" s="27"/>
+      <c r="K69" s="24"/>
+      <c r="L69" s="104"/>
+      <c r="V69" s="1"/>
+      <c r="W69" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M70" s="37"/>
+      <c r="N70" s="38"/>
+      <c r="O70" s="39"/>
+      <c r="P70" s="151">
+        <v>605671</v>
+      </c>
+      <c r="Q70" s="65">
+        <v>10016</v>
+      </c>
+      <c r="R70" s="153"/>
+      <c r="S70" s="73"/>
+      <c r="T70" s="151"/>
+      <c r="U70" s="67"/>
+      <c r="A70" s="1"/>
+      <c r="I70" s="108"/>
+      <c r="J70" s="27"/>
+      <c r="K70" s="24"/>
+      <c r="L70" s="104"/>
+      <c r="V70" s="1"/>
+      <c r="W70" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B71" s="20"/>
+      <c r="C71" s="32"/>
+      <c r="I71" s="108">
+        <f>M$1</f>
+        <v>0</v>
+      </c>
+      <c r="J71" s="27">
+        <f t="shared" ref="J71:J78" si="6">L10</f>
+        <v>0</v>
+      </c>
+      <c r="L71" s="104"/>
+      <c r="M71" s="202" t="s">
+        <v>42</v>
+      </c>
+      <c r="N71" s="203"/>
+      <c r="O71" s="149"/>
+      <c r="P71" s="151"/>
+      <c r="Q71" s="74"/>
+      <c r="R71" s="153"/>
+      <c r="S71" s="72"/>
+      <c r="T71" s="151"/>
+      <c r="U71" s="75"/>
+      <c r="V71" s="1"/>
+      <c r="W71" s="1"/>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M72" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30-07-2026</t>
+        </is>
+      </c>
+      <c r="N72" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCI</t>
+        </is>
+      </c>
+      <c r="O72" s="39">
+        <v>127092</v>
+      </c>
+      <c r="B72" s="20"/>
+      <c r="C72" s="32"/>
+      <c r="I72" s="108">
+        <f>N$1</f>
+        <v>0</v>
+      </c>
+      <c r="J72" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="M73" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30-07-2026</t>
+        </is>
+      </c>
+      <c r="N73" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCI</t>
+        </is>
+      </c>
+      <c r="O73" s="39">
+        <v>972618</v>
+      </c>
+      <c r="J73" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M74" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30-07-2026</t>
+        </is>
+      </c>
+      <c r="N74" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCI</t>
+        </is>
+      </c>
+      <c r="O74" s="39">
+        <v>368449</v>
+      </c>
+      <c r="J74" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="M75" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30-07-2026</t>
+        </is>
+      </c>
+      <c r="N75" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCI</t>
+        </is>
+      </c>
+      <c r="O75" s="39">
+        <v>92552</v>
+      </c>
+      <c r="J75" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="J76" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J77" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="J78" s="27">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="L79" s="104"/>
+      <c r="M79" s="37"/>
+      <c r="N79" s="38"/>
+      <c r="O79" s="39"/>
+      <c r="P79" s="151"/>
+      <c r="Q79" s="65"/>
+      <c r="R79" s="151"/>
+      <c r="S79" s="66"/>
+      <c r="T79" s="151"/>
+      <c r="U79" s="67"/>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A80" s="20"/>
+      <c r="B80" s="20"/>
+      <c r="C80" s="40"/>
+      <c r="D80" s="192"/>
+      <c r="E80" s="192"/>
+      <c r="F80" s="17"/>
+      <c r="G80" s="1"/>
+      <c r="H80" s="63"/>
+      <c r="I80" s="13"/>
+      <c r="J80" s="52"/>
+      <c r="K80" s="24"/>
+      <c r="L80" s="104"/>
+      <c r="M80" s="37"/>
+      <c r="N80" s="38"/>
+      <c r="O80" s="39"/>
+      <c r="P80" s="151"/>
+      <c r="Q80" s="65"/>
+      <c r="R80" s="151"/>
+      <c r="S80" s="66"/>
+      <c r="T80" s="151"/>
+      <c r="U80" s="67"/>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A81" s="20"/>
+      <c r="B81" s="20"/>
+      <c r="C81" s="40"/>
+      <c r="D81" s="192"/>
+      <c r="E81" s="192"/>
+      <c r="F81" s="23"/>
+      <c r="G81" s="1"/>
+      <c r="H81" s="63"/>
+      <c r="I81" s="13"/>
+      <c r="J81" s="52"/>
+      <c r="L81" s="104"/>
+      <c r="M81" s="37"/>
+      <c r="N81" s="38"/>
+      <c r="O81" s="39"/>
+      <c r="P81" s="151"/>
+      <c r="Q81" s="65"/>
+      <c r="R81" s="151"/>
+      <c r="S81" s="66"/>
+      <c r="T81" s="153"/>
+      <c r="U81" s="67"/>
+    </row>
+    <row r="82" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A82" s="20"/>
+      <c r="B82" s="20"/>
+      <c r="C82" s="40"/>
+      <c r="D82" s="192"/>
+      <c r="E82" s="192"/>
+      <c r="F82" s="23"/>
+      <c r="G82" s="1"/>
+      <c r="H82" s="45"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="52"/>
+      <c r="L82" s="104"/>
+      <c r="M82" s="37"/>
+      <c r="N82" s="38"/>
+      <c r="O82" s="39"/>
+      <c r="P82" s="151"/>
+      <c r="Q82" s="65"/>
+      <c r="R82" s="151"/>
+      <c r="S82" s="66"/>
+      <c r="T82" s="153"/>
+      <c r="U82" s="67"/>
+    </row>
+    <row r="83" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A83" s="20"/>
+      <c r="B83" s="20"/>
+      <c r="C83" s="40"/>
+      <c r="D83" s="23"/>
+      <c r="E83" s="25"/>
+      <c r="F83" s="23"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="45"/>
+      <c r="I83" s="13"/>
+      <c r="J83" s="52"/>
+      <c r="L83" s="104"/>
+      <c r="M83" s="37"/>
+      <c r="N83" s="38"/>
+      <c r="O83" s="39"/>
+      <c r="P83" s="151"/>
+      <c r="Q83" s="65"/>
+      <c r="R83" s="151"/>
+      <c r="S83" s="66"/>
+      <c r="T83" s="153"/>
+      <c r="U83" s="67"/>
+    </row>
+    <row r="84" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A84" s="20"/>
+      <c r="B84" s="20"/>
+      <c r="C84" s="40"/>
+      <c r="D84" s="218"/>
+      <c r="E84" s="218"/>
+      <c r="F84" s="23"/>
+      <c r="G84" s="1"/>
+      <c r="H84" s="45"/>
+      <c r="I84" s="13"/>
+      <c r="J84" s="52"/>
+      <c r="L84" s="104"/>
+      <c r="M84" s="37"/>
+      <c r="N84" s="38"/>
+      <c r="O84" s="39"/>
+      <c r="P84" s="150"/>
+      <c r="Q84" s="65"/>
+      <c r="R84" s="151"/>
+      <c r="S84" s="66"/>
+      <c r="T84" s="153"/>
+      <c r="U84" s="67"/>
+    </row>
+    <row r="85" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A85" s="20"/>
+      <c r="B85" s="50"/>
+      <c r="C85" s="40"/>
+      <c r="D85" s="205"/>
+      <c r="E85" s="205"/>
+      <c r="F85" s="23"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="45"/>
+      <c r="I85" s="49"/>
+      <c r="J85" s="52"/>
+      <c r="L85" s="104"/>
+      <c r="M85" s="37"/>
+      <c r="N85" s="38"/>
+      <c r="O85" s="39"/>
+      <c r="P85" s="150"/>
+      <c r="Q85" s="65"/>
+      <c r="R85" s="151"/>
+      <c r="S85" s="66"/>
+      <c r="T85" s="153"/>
+      <c r="U85" s="67"/>
+    </row>
+    <row r="86" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A86" s="25"/>
+      <c r="B86" s="50"/>
+      <c r="C86" s="40"/>
+      <c r="D86" s="204"/>
+      <c r="E86" s="204"/>
+      <c r="F86" s="23"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="45"/>
+      <c r="I86" s="49"/>
+      <c r="J86" s="52"/>
+      <c r="L86" s="18"/>
+      <c r="M86" s="37"/>
+      <c r="N86" s="38"/>
+      <c r="O86" s="39"/>
+      <c r="P86" s="151"/>
+      <c r="Q86" s="65"/>
+      <c r="R86" s="151"/>
+      <c r="S86" s="66"/>
+      <c r="T86" s="153"/>
+      <c r="U86" s="67"/>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A87" s="20"/>
+      <c r="B87" s="50"/>
+      <c r="C87" s="40"/>
+      <c r="D87" s="204"/>
+      <c r="E87" s="204"/>
+      <c r="F87" s="23"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="45"/>
+      <c r="I87" s="49"/>
+      <c r="J87" s="52"/>
+      <c r="L87" s="18"/>
+      <c r="M87" s="37"/>
+      <c r="N87" s="38"/>
+      <c r="O87" s="39"/>
+      <c r="P87" s="151"/>
+      <c r="Q87" s="65"/>
+      <c r="R87" s="151"/>
+      <c r="S87" s="66"/>
+      <c r="T87" s="153"/>
+      <c r="U87" s="67"/>
+    </row>
+    <row r="88" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A88" s="20"/>
+      <c r="B88" s="50"/>
+      <c r="C88" s="40"/>
+      <c r="D88" s="22"/>
+      <c r="E88" s="22"/>
+      <c r="F88" s="23"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="45"/>
+      <c r="I88" s="49"/>
+      <c r="J88" s="52"/>
+      <c r="L88" s="18"/>
+      <c r="M88" s="37"/>
+      <c r="N88" s="38"/>
+      <c r="O88" s="39"/>
+      <c r="P88" s="151"/>
+      <c r="Q88" s="65"/>
+      <c r="R88" s="151"/>
+      <c r="S88" s="66"/>
+      <c r="T88" s="153"/>
+      <c r="U88" s="67"/>
+    </row>
+    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A89" s="20"/>
+      <c r="B89"/>
+      <c r="C89" s="40"/>
+      <c r="D89" s="22"/>
+      <c r="E89" s="22"/>
+      <c r="F89" s="23"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="45"/>
+      <c r="I89" s="49"/>
+      <c r="J89" s="52"/>
+      <c r="L89" s="18"/>
+      <c r="M89" s="37"/>
+      <c r="N89" s="38"/>
+      <c r="O89" s="39"/>
+      <c r="P89" s="151"/>
+      <c r="Q89" s="65"/>
+      <c r="R89" s="151"/>
+      <c r="S89" s="66"/>
+      <c r="T89" s="153"/>
+      <c r="U89" s="67"/>
+    </row>
+    <row r="90" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A90" s="20"/>
+      <c r="B90"/>
+      <c r="C90" s="40"/>
+      <c r="D90" s="22"/>
+      <c r="E90" s="22"/>
+      <c r="F90" s="23"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="45"/>
+      <c r="I90" s="49"/>
+      <c r="J90" s="52"/>
+      <c r="L90" s="18"/>
+      <c r="M90" s="37"/>
+      <c r="N90" s="38"/>
+      <c r="O90" s="39"/>
+      <c r="P90" s="151"/>
+      <c r="Q90" s="65"/>
+      <c r="R90" s="151"/>
+      <c r="S90" s="66"/>
+      <c r="T90" s="153"/>
+      <c r="U90" s="67"/>
+    </row>
+    <row r="91" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A91" s="20"/>
+      <c r="B91"/>
+      <c r="C91" s="40"/>
+      <c r="D91" s="22"/>
+      <c r="E91" s="22"/>
+      <c r="F91" s="23"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="45"/>
+      <c r="I91" s="49"/>
+      <c r="J91" s="52"/>
+      <c r="L91" s="18"/>
+      <c r="M91" s="37"/>
+      <c r="N91" s="38"/>
+      <c r="O91" s="39"/>
+      <c r="P91" s="151"/>
+      <c r="Q91" s="65"/>
+      <c r="R91" s="151"/>
+      <c r="S91" s="66"/>
+      <c r="T91" s="153"/>
+      <c r="U91" s="67"/>
+    </row>
+    <row r="92" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A92" s="20"/>
+      <c r="B92"/>
+      <c r="C92" s="40"/>
+      <c r="D92" s="22"/>
+      <c r="E92" s="22"/>
+      <c r="F92" s="23"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="45"/>
+      <c r="I92" s="49"/>
+      <c r="J92" s="52"/>
+      <c r="L92" s="18"/>
+      <c r="M92" s="37"/>
+      <c r="N92" s="38"/>
+      <c r="O92" s="39"/>
+      <c r="P92" s="151"/>
+      <c r="Q92" s="65"/>
+      <c r="R92" s="151"/>
+      <c r="S92" s="66"/>
+      <c r="T92" s="153"/>
+      <c r="U92" s="67"/>
+    </row>
+    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A93" s="25"/>
+      <c r="B93"/>
+      <c r="C93" s="40"/>
+      <c r="D93" s="204"/>
+      <c r="E93" s="204"/>
+      <c r="F93" s="23"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="45"/>
+      <c r="I93" s="49"/>
+      <c r="J93" s="52"/>
+      <c r="L93" s="18"/>
+      <c r="M93" s="37"/>
+      <c r="N93" s="38"/>
+      <c r="O93" s="39"/>
+      <c r="P93" s="151"/>
+      <c r="Q93" s="65"/>
+      <c r="R93" s="151"/>
+      <c r="S93" s="66"/>
+      <c r="T93" s="153"/>
+      <c r="U93" s="67"/>
+    </row>
+    <row r="94" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A94" s="25"/>
+      <c r="B94"/>
+      <c r="C94" s="40"/>
+      <c r="D94" s="22"/>
+      <c r="E94" s="22"/>
+      <c r="F94" s="23"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="45"/>
+      <c r="I94" s="49"/>
+      <c r="J94" s="52"/>
+      <c r="L94" s="18"/>
+      <c r="M94" s="37"/>
+      <c r="N94" s="38"/>
+      <c r="O94" s="39"/>
+      <c r="P94" s="151"/>
+      <c r="Q94" s="134"/>
+      <c r="R94" s="154"/>
+      <c r="S94" s="87"/>
+      <c r="T94" s="153"/>
+      <c r="U94" s="67"/>
+    </row>
+    <row r="95" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A95" s="25"/>
+      <c r="B95"/>
+      <c r="C95" s="40"/>
+      <c r="D95" s="22"/>
+      <c r="E95" s="22"/>
+      <c r="F95" s="23"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="45"/>
+      <c r="I95" s="49"/>
+      <c r="J95" s="52"/>
+      <c r="L95" s="18"/>
+      <c r="M95" s="37"/>
+      <c r="N95" s="38"/>
+      <c r="O95" s="39"/>
+      <c r="P95" s="151"/>
+      <c r="Q95" s="134"/>
+      <c r="R95" s="154"/>
+      <c r="S95" s="87"/>
+      <c r="T95" s="153"/>
+      <c r="U95" s="67"/>
+    </row>
+    <row r="96" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A96" s="25"/>
+      <c r="B96"/>
+      <c r="C96" s="40"/>
+      <c r="D96" s="22"/>
+      <c r="E96" s="22"/>
+      <c r="F96" s="23"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="45"/>
+      <c r="I96" s="49"/>
+      <c r="J96" s="52"/>
+      <c r="L96" s="18"/>
+      <c r="M96" s="37"/>
+      <c r="N96" s="38"/>
+      <c r="O96" s="39"/>
+      <c r="P96" s="151"/>
+      <c r="Q96" s="134"/>
+      <c r="R96" s="154"/>
+      <c r="S96" s="87"/>
+      <c r="T96" s="153"/>
+      <c r="U96" s="67"/>
+    </row>
+    <row r="97" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A97" s="25"/>
+      <c r="B97"/>
+      <c r="C97" s="40"/>
+      <c r="D97" s="204"/>
+      <c r="E97" s="204"/>
+      <c r="F97" s="23"/>
+      <c r="G97" s="1"/>
+      <c r="H97" s="45"/>
+      <c r="I97" s="49"/>
+      <c r="J97" s="52"/>
+      <c r="L97" s="18"/>
+      <c r="M97" s="37"/>
+      <c r="N97" s="38"/>
+      <c r="O97" s="39"/>
+      <c r="P97" s="151"/>
+      <c r="Q97" s="83"/>
+      <c r="R97" s="154"/>
+      <c r="S97" s="87"/>
+      <c r="T97" s="153"/>
+      <c r="U97" s="70"/>
+    </row>
+    <row r="98" spans="1:23" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="25"/>
+      <c r="B98"/>
+      <c r="C98" s="40"/>
+      <c r="D98" s="204"/>
+      <c r="E98" s="204"/>
+      <c r="F98" s="20"/>
+      <c r="G98" s="1"/>
+      <c r="H98" s="45"/>
+      <c r="I98" s="49"/>
+      <c r="J98" s="52"/>
+      <c r="L98"/>
+      <c r="M98" s="202" t="s">
+        <v>34</v>
+      </c>
+      <c r="N98" s="217"/>
+      <c r="O98" s="41">
+        <v>1560711</v>
+      </c>
+      <c r="P98" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q98" s="41"/>
+      <c r="R98" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="S98" s="41"/>
+      <c r="T98" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="U98" s="41"/>
+    </row>
+    <row r="99" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A99" s="25"/>
+      <c r="B99"/>
+      <c r="C99" s="89"/>
+      <c r="D99" s="204"/>
+      <c r="E99" s="204"/>
+      <c r="F99" s="23"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="45"/>
+      <c r="I99" s="49"/>
+      <c r="J99"/>
+      <c r="L99"/>
+      <c r="M99" s="53"/>
+      <c r="N99" s="54"/>
+      <c r="O99" s="69"/>
+      <c r="P99" s="23"/>
+      <c r="Q99" s="68"/>
+      <c r="R99" s="69"/>
+      <c r="S99" s="69"/>
+      <c r="T99" s="6"/>
+    </row>
+    <row r="100" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A100" s="25"/>
+      <c r="B100"/>
+      <c r="C100" s="25"/>
+      <c r="D100" s="22"/>
+      <c r="E100" s="22"/>
+      <c r="F100" s="23"/>
+      <c r="G100" s="1"/>
+      <c r="H100" s="45"/>
+      <c r="I100" s="49"/>
+      <c r="J100"/>
+      <c r="L100"/>
+      <c r="M100" s="193" t="s">
+        <v>47</v>
+      </c>
+      <c r="N100" s="207"/>
+      <c r="O100" s="194"/>
+      <c r="P100" s="208"/>
+      <c r="Q100" s="209"/>
+      <c r="R100" s="193" t="s">
+        <v>37</v>
+      </c>
+      <c r="S100" s="207"/>
+      <c r="T100" s="210" t="str">
+        <f>Q25</f>
+      </c>
+      <c r="U100" s="211"/>
+    </row>
+    <row r="101" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A101" s="25"/>
+      <c r="B101"/>
+      <c r="C101" s="25"/>
+      <c r="D101" s="204"/>
+      <c r="E101" s="204"/>
+      <c r="F101" s="62"/>
+      <c r="G101" s="1"/>
+      <c r="H101" s="45"/>
+      <c r="I101" s="49"/>
+      <c r="J101"/>
+      <c r="L101"/>
+      <c r="M101" s="55"/>
+      <c r="N101" s="82"/>
+      <c r="O101" s="82"/>
+      <c r="P101" s="56"/>
+      <c r="Q101" s="57"/>
+      <c r="R101" s="57"/>
+      <c r="S101" s="57"/>
+      <c r="T101" s="55"/>
+      <c r="U101" s="55"/>
+    </row>
+    <row r="102" spans="1:23" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="25"/>
+      <c r="B102" s="89"/>
+      <c r="C102" s="25"/>
+      <c r="D102" s="204"/>
+      <c r="E102" s="204"/>
+      <c r="F102" s="62"/>
+      <c r="G102" s="1"/>
+      <c r="H102" s="45"/>
+      <c r="I102" s="49"/>
+      <c r="J102"/>
+      <c r="L102"/>
+      <c r="M102" s="202" t="s">
+        <v>35</v>
+      </c>
+      <c r="N102" s="203"/>
+      <c r="O102" s="203"/>
+      <c r="P102" s="203"/>
+      <c r="Q102" s="203"/>
+      <c r="R102" s="203"/>
+      <c r="S102" s="203"/>
+      <c r="T102" s="203"/>
+      <c r="U102" s="206"/>
+      <c r="V102" s="50"/>
+    </row>
+    <row r="103" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A103" s="25"/>
+      <c r="B103" s="20"/>
+      <c r="C103" s="25"/>
+      <c r="D103" s="204"/>
+      <c r="E103" s="204"/>
+      <c r="F103" s="62"/>
+      <c r="G103" s="1"/>
+      <c r="H103" s="45"/>
+      <c r="I103" s="49"/>
+      <c r="J103"/>
+      <c r="L103" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="M103" s="129" t="s">
+        <v>55</v>
+      </c>
+      <c r="N103" s="130"/>
+      <c r="O103" s="130"/>
+      <c r="P103" s="130" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q103" s="130"/>
+      <c r="R103" s="130"/>
+      <c r="S103" s="130"/>
+      <c r="T103" s="130" t="s">
+        <v>57</v>
+      </c>
+      <c r="U103" s="131" t="s">
+        <v>60</v>
+      </c>
+      <c r="V103" s="143" t="s">
+        <v>58</v>
+      </c>
+      <c r="W103" s="143" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L104" s="0"/>
+      <c r="M104" s="58"/>
+      <c r="P104" s="61"/>
+      <c r="T104" s="132"/>
+      <c r="V104" s="50"/>
+      <c r="R104" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CREDITO</t>
+        </is>
+      </c>
+      <c r="A104" s="25"/>
+      <c r="B104" s="114"/>
+      <c r="C104" s="25"/>
+      <c r="D104" s="204"/>
+      <c r="E104" s="204"/>
+      <c r="F104" s="62"/>
+      <c r="G104" s="1"/>
+      <c r="H104" s="45"/>
+      <c r="I104" s="49"/>
+      <c r="J104" s="23"/>
+      <c r="N104" s="59"/>
+      <c r="O104" s="142" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q104" s="60"/>
+      <c r="S104" s="216"/>
+      <c r="U104" s="133"/>
+    </row>
+    <row r="105" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B105" s="50"/>
+      <c r="C105" s="88"/>
+      <c r="D105" s="204"/>
+      <c r="E105" s="204"/>
+      <c r="F105" s="62"/>
+      <c r="I105" s="114"/>
+      <c r="L105"/>
+      <c r="M105" s="84"/>
+      <c r="N105" s="85"/>
+      <c r="O105" s="18"/>
+      <c r="P105" s="86"/>
+      <c r="Q105" s="55"/>
+      <c r="R105" s="214"/>
+      <c r="S105" s="214"/>
+      <c r="T105" s="64"/>
+      <c r="U105" s="94"/>
+      <c r="V105" s="50"/>
+    </row>
+    <row r="106" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L106" s="44"/>
+      <c r="M106" s="84"/>
+      <c r="P106" s="86"/>
+      <c r="T106" s="64"/>
+      <c r="U106" s="94"/>
+      <c r="R106" s="214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRANSFERENCIA</t>
+        </is>
+      </c>
+      <c r="A106" s="48"/>
+      <c r="B106" s="88"/>
+      <c r="C106" s="88"/>
+      <c r="D106" s="23"/>
+      <c r="E106" s="25"/>
+      <c r="F106" s="62"/>
+      <c r="I106" s="114"/>
+      <c r="N106" s="85"/>
+      <c r="O106" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q106" s="55"/>
+      <c r="S106" s="214"/>
+      <c r="V106" s="50"/>
+    </row>
+    <row r="107" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L107" s="44"/>
+      <c r="M107" s="84"/>
+      <c r="N107" s="85"/>
+      <c r="O107" s="122"/>
+      <c r="P107" s="86"/>
+      <c r="Q107" s="55"/>
+      <c r="R107" s="214"/>
+      <c r="S107" s="214"/>
+      <c r="T107" s="64"/>
+      <c r="U107" s="94"/>
+      <c r="V107" s="50"/>
+    </row>
+    <row r="108" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L108" s="44"/>
+      <c r="M108" s="136" t="s">
+        <v>61</v>
+      </c>
+      <c r="N108" s="137"/>
+      <c r="O108" s="138"/>
+      <c r="P108" s="139"/>
+      <c r="Q108" s="140"/>
+      <c r="R108" s="215"/>
+      <c r="S108" s="215"/>
+      <c r="T108" s="212"/>
+      <c r="U108" s="213"/>
+      <c r="V108" s="50"/>
+    </row>
+    <row r="109" spans="1:23" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="L109" s="44"/>
+      <c r="M109" s="136" t="s">
+        <v>62</v>
+      </c>
+      <c r="N109" s="137"/>
+      <c r="O109" s="138"/>
+      <c r="P109" s="139"/>
+      <c r="Q109" s="140"/>
+      <c r="R109" s="141"/>
+      <c r="S109" s="141"/>
+      <c r="T109" s="212"/>
+      <c r="U109" s="213"/>
+      <c r="V109" s="50"/>
+    </row>
+    <row r="110" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L110" s="44"/>
+      <c r="M110" s="93"/>
+      <c r="N110" s="63"/>
+      <c r="O110" s="122"/>
+      <c r="P110" s="86"/>
+      <c r="Q110" s="55"/>
+      <c r="R110" s="55"/>
+      <c r="S110" s="55"/>
+      <c r="T110" s="64"/>
+      <c r="U110" s="94"/>
+      <c r="V110" s="50"/>
+    </row>
+    <row r="111" spans="1:23" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L111" s="44"/>
+      <c r="M111" s="100" t="s">
+        <v>11</v>
+      </c>
+      <c r="N111" s="101">
+        <f>SUM(N109:N110)</f>
+        <v>0</v>
+      </c>
+      <c r="O111" s="95"/>
+      <c r="P111" s="97"/>
+      <c r="Q111" s="96"/>
+      <c r="R111" s="96"/>
+      <c r="S111" s="96"/>
+      <c r="T111" s="98"/>
+      <c r="U111" s="99"/>
+      <c r="V111" s="50"/>
+    </row>
+    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="M112"/>
+      <c r="O112" s="5"/>
+      <c r="Q112"/>
+      <c r="S112"/>
+      <c r="T112" s="6"/>
+      <c r="V112" s="50"/>
+    </row>
+    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="O113"/>
+      <c r="V113" s="50"/>
+    </row>
+    <row r="114" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="M114" s="23"/>
+      <c r="N114" s="23"/>
+      <c r="O114" s="23"/>
+      <c r="P114" s="23"/>
+      <c r="Q114" s="23"/>
+      <c r="V114" s="50"/>
+    </row>
+    <row r="115" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V115" s="50"/>
+    </row>
+    <row r="116" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V116" s="50"/>
+    </row>
+    <row r="117" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V117" s="50"/>
+    </row>
+    <row r="118" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V118" s="50"/>
+    </row>
+    <row r="119" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V119" s="50"/>
+    </row>
+    <row r="120" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V120" s="50"/>
+    </row>
+    <row r="121" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V121" s="50"/>
+    </row>
+    <row r="122" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V122" s="50"/>
+    </row>
+    <row r="123" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V123" s="50"/>
+    </row>
+    <row r="124" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V124" s="50"/>
+    </row>
+    <row r="125" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V125" s="50"/>
+    </row>
+    <row r="126" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V126" s="50"/>
+    </row>
+    <row r="127" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V127" s="50"/>
+    </row>
+    <row r="128" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V128" s="50"/>
+    </row>
+    <row r="129" spans="13:22" x14ac:dyDescent="0.3">
+      <c r="V129" s="50"/>
+    </row>
+    <row r="130" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V130" s="50"/>
+    </row>
+    <row r="131" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V131" s="50"/>
+    </row>
+    <row r="132" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V132" s="50"/>
+    </row>
+    <row r="133" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V133" s="50"/>
+    </row>
+    <row r="134" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V134" s="50"/>
+    </row>
+    <row r="135" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V135" s="50"/>
+    </row>
+    <row r="136" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V136" s="50"/>
+    </row>
+    <row r="137" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V137" s="50"/>
+    </row>
+    <row r="138" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V138" s="50"/>
+    </row>
+    <row r="139" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V139" s="50"/>
+    </row>
+    <row r="140" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V140" s="50"/>
+    </row>
+    <row r="141" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V141" s="50"/>
+    </row>
+    <row r="142" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V142" s="50"/>
+    </row>
+    <row r="143" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V143" s="50"/>
+    </row>
+    <row r="144" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V144" s="50"/>
+    </row>
+    <row r="145" spans="22:22" x14ac:dyDescent="0.3">
+      <c r="V145" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells count="70">
+    <mergeCell ref="M100:O100"/>
+    <mergeCell ref="D77:E77"/>
+    <mergeCell ref="D79:E79"/>
+    <mergeCell ref="M98:N98"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="D78:E78"/>
+    <mergeCell ref="D84:E84"/>
+    <mergeCell ref="T109:U109"/>
+    <mergeCell ref="R107:S107"/>
+    <mergeCell ref="R108:S108"/>
+    <mergeCell ref="R104:S104"/>
+    <mergeCell ref="R106:S106"/>
+    <mergeCell ref="R105:S105"/>
+    <mergeCell ref="T108:U108"/>
+    <mergeCell ref="D104:E104"/>
+    <mergeCell ref="D105:E105"/>
+    <mergeCell ref="D85:E85"/>
+    <mergeCell ref="M102:U102"/>
+    <mergeCell ref="R100:S100"/>
+    <mergeCell ref="D101:E101"/>
+    <mergeCell ref="P100:Q100"/>
+    <mergeCell ref="T100:U100"/>
+    <mergeCell ref="D93:E93"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="D98:E98"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="D97:E97"/>
+    <mergeCell ref="D103:E103"/>
+    <mergeCell ref="D102:E102"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:S33"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:S34"/>
+    <mergeCell ref="P35:Q35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M71:N71"/>
+    <mergeCell ref="M22:U22"/>
+    <mergeCell ref="Q26:S26"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="Q29:S29"/>
+    <mergeCell ref="T29:U29"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="Q28:S28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="Q27:S27"/>
+    <mergeCell ref="T27:U27"/>
+    <mergeCell ref="N23:S23"/>
+    <mergeCell ref="N24:S24"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="M25:N25"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="Q30:S30"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="Q32:S32"/>
+    <mergeCell ref="M31:N31"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="Q31:S31"/>
+    <mergeCell ref="M30:N30"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="O32:P32"/>
+  </mergeCells>
+  <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="5" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>